<commit_message>
docs(testes): adicionar TC-FLUXO-03 e TC-FLUXO-04 ao plano v3.40.0 (BUG-033 #216, BUG-034 #217)
</commit_message>
<xml_diff>
--- a/docs/PLANO_DE_TESTES_v3.40.0.xlsx
+++ b/docs/PLANO_DE_TESTES_v3.40.0.xlsx
@@ -143,7 +143,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -166,6 +166,50 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1">
@@ -177,7 +221,7 @@
     <xf numFmtId="42" fontId="3" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="39">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
@@ -281,6 +325,8 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="general" vertical="bottom"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -671,7 +717,7 @@
       </c>
       <c r="B6" s="20" t="inlineStr">
         <is>
-          <t>Full UAT — Regressao v3.39.8 + Novos v3.40.0 (Polimento Visual: ENH-007 + RF-071 + ENH-006)</t>
+          <t>Full UAT — Regressao v3.39.8 + Novos v3.40.0 (Polimento Visual: ENH-007 + RF-071 + ENH-006) + Regressao pos-UAT (BUG-033 #216, BUG-034 #217)</t>
         </is>
       </c>
     </row>
@@ -683,7 +729,7 @@
       </c>
       <c r="B7" s="20" t="inlineStr">
         <is>
-          <t>Full — 98 TCs (85 herdados de v3.39.8 + 13 novos de v3.40.0)</t>
+          <t>Full — 100 TCs (85 herdados de v3.39.8 + 13 Polimento Visual + 2 Regressao pos-UAT)</t>
         </is>
       </c>
     </row>
@@ -789,7 +835,7 @@
       <c r="A21" s="20" t="n"/>
       <c r="B21" s="20" t="inlineStr">
         <is>
-          <t>[ ] 98/98 TCs com status PASS ou N/A justificado</t>
+          <t>[ ] 100/100 TCs com status PASS ou N/A justificado</t>
         </is>
       </c>
     </row>
@@ -886,7 +932,11 @@
     </row>
     <row r="34" ht="15" customHeight="1" s="18">
       <c r="A34" s="20" t="n"/>
-      <c r="B34" s="20" t="n"/>
+      <c r="B34" s="20" t="inlineStr">
+        <is>
+          <t>Regressao pos-UAT v3.40.0: 2 TCs (TC-FLUXO-03 BUG-033 #216 + TC-FLUXO-04 BUG-034 #217)</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="15" customHeight="1" s="18">
       <c r="A35" s="20" t="n"/>
@@ -927,7 +977,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:M125"/>
+  <dimension ref="A1:M128"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="5" customWidth="1" style="17" min="1" max="1"/>
@@ -946,7 +996,7 @@
     <row r="1" ht="27.75" customHeight="1" s="18">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>Casos de Teste v3.40.0 — Full UAT (98 TCs)</t>
+          <t>Casos de Teste v3.40.0 — Full UAT (100 TCs) + Regressao pos-UAT</t>
         </is>
       </c>
     </row>
@@ -1018,63 +1068,63 @@
       </c>
     </row>
     <row r="3" ht="45.75" customHeight="1" s="18">
-      <c r="A3" s="24" t="n">
+      <c r="A3" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B3" s="24" t="inlineStr">
+      <c r="B3" s="27" t="inlineStr">
         <is>
           <t>TC-AUTH-01</t>
         </is>
       </c>
-      <c r="C3" s="24" t="inlineStr">
+      <c r="C3" s="27" t="inlineStr">
         <is>
           <t>Auth</t>
         </is>
       </c>
-      <c r="D3" s="25" t="inlineStr">
+      <c r="D3" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E3" s="24" t="inlineStr">
+      <c r="E3" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F3" s="24" t="inlineStr">
+      <c r="F3" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G3" s="24" t="inlineStr">
+      <c r="G3" s="27" t="inlineStr">
         <is>
           <t>Login Luigi com email/senha</t>
         </is>
       </c>
-      <c r="H3" s="24" t="inlineStr">
+      <c r="H3" s="27" t="inlineStr">
         <is>
           <t>1. Abrir /login.html
 2. Preencher email e senha
 3. Clicar em Entrar</t>
         </is>
       </c>
-      <c r="I3" s="24" t="inlineStr">
+      <c r="I3" s="27" t="inlineStr">
         <is>
           <t>Redireciona para /dashboard.html; navbar exibe nome do usuario; sessao persiste em refresh</t>
         </is>
       </c>
-      <c r="J3" s="24" t="inlineStr">
+      <c r="J3" s="27" t="inlineStr">
         <is>
           <t>CLAUDE.md - onAuthChange</t>
         </is>
       </c>
-      <c r="K3" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L3" s="24" t="n"/>
-      <c r="M3" s="24" t="n"/>
+      <c r="K3" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L3" s="27" t="n"/>
+      <c r="M3" s="27" t="n"/>
     </row>
     <row r="4" ht="45" customHeight="1" s="18">
       <c r="A4" s="26" t="n">
@@ -1135,63 +1185,63 @@
       <c r="M4" s="26" t="n"/>
     </row>
     <row r="5" ht="45.75" customHeight="1" s="18">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>TC-NAV-01</t>
         </is>
       </c>
-      <c r="C5" s="24" t="inlineStr">
+      <c r="C5" s="27" t="inlineStr">
         <is>
           <t>Navegacao</t>
         </is>
       </c>
-      <c r="D5" s="25" t="inlineStr">
+      <c r="D5" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E5" s="24" t="inlineStr">
+      <c r="E5" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F5" s="24" t="inlineStr">
+      <c r="F5" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G5" s="24" t="inlineStr">
+      <c r="G5" s="27" t="inlineStr">
         <is>
           <t>Navbar 5 secoes expande Cockpit corretamente</t>
         </is>
       </c>
-      <c r="H5" s="24" t="inlineStr">
+      <c r="H5" s="27" t="inlineStr">
         <is>
           <t>1. Abrir /dashboard.html
 2. Observar secao Cockpit aberta com Dashboard + Planejamento
 3. Clicar em outras secoes (Historico, Transacoes, Futuro, Config)</t>
         </is>
       </c>
-      <c r="I5" s="24" t="inlineStr">
+      <c r="I5" s="27" t="inlineStr">
         <is>
           <t>Somente secao ativa fica aberta; sub-item ativo marcado; sem JS errors no console</t>
         </is>
       </c>
-      <c r="J5" s="24" t="inlineStr">
+      <c r="J5" s="27" t="inlineStr">
         <is>
           <t>src/js/nav.js sectionMap</t>
         </is>
       </c>
-      <c r="K5" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L5" s="24" t="n"/>
-      <c r="M5" s="24" t="n"/>
+      <c r="K5" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L5" s="27" t="n"/>
+      <c r="M5" s="27" t="n"/>
     </row>
     <row r="6" ht="45" customHeight="1" s="18">
       <c r="A6" s="26" t="n">
@@ -1252,62 +1302,62 @@
       <c r="M6" s="26" t="n"/>
     </row>
     <row r="7" ht="45" customHeight="1" s="18">
-      <c r="A7" s="24" t="n">
+      <c r="A7" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>TC-NAV-03</t>
         </is>
       </c>
-      <c r="C7" s="24" t="inlineStr">
+      <c r="C7" s="27" t="inlineStr">
         <is>
           <t>Navegacao</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E7" s="24" t="inlineStr">
+      <c r="E7" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F7" s="24" t="inlineStr">
+      <c r="F7" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G7" s="24" t="inlineStr">
+      <c r="G7" s="27" t="inlineStr">
         <is>
           <t>Deep-link fatura?tab=projecoes ativa secao Futuro</t>
         </is>
       </c>
-      <c r="H7" s="24" t="inlineStr">
+      <c r="H7" s="27" t="inlineStr">
         <is>
           <t>1. Acessar diretamente /fatura.html?tab=projecoes
 2. Observar qual secao da navbar abre</t>
         </is>
       </c>
-      <c r="I7" s="24" t="inlineStr">
+      <c r="I7" s="27" t="inlineStr">
         <is>
           <t>Secao Futuro aberta (nao Transacoes) + sub-item Fluxo de Caixa destacado</t>
         </is>
       </c>
-      <c r="J7" s="24" t="inlineStr">
+      <c r="J7" s="27" t="inlineStr">
         <is>
           <t>nav.js linha branch especial tab=projecoes</t>
         </is>
       </c>
-      <c r="K7" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L7" s="24" t="n"/>
-      <c r="M7" s="24" t="n"/>
+      <c r="K7" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L7" s="27" t="n"/>
+      <c r="M7" s="27" t="n"/>
     </row>
     <row r="8" ht="45.75" customHeight="1" s="18">
       <c r="A8" s="26" t="n">
@@ -1323,7 +1373,7 @@
           <t>Cockpit/Dashboard</t>
         </is>
       </c>
-      <c r="D8" s="25" t="inlineStr">
+      <c r="D8" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1369,62 +1419,62 @@
       <c r="M8" s="26" t="n"/>
     </row>
     <row r="9" ht="45" customHeight="1" s="18">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>TC-DASH-02</t>
         </is>
       </c>
-      <c r="C9" s="24" t="inlineStr">
+      <c r="C9" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Dashboard</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E9" s="24" t="inlineStr">
+      <c r="E9" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F9" s="24" t="inlineStr">
+      <c r="F9" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G9" s="24" t="inlineStr">
+      <c r="G9" s="27" t="inlineStr">
         <is>
           <t>Saldo Real por conta reflete contas ativas</t>
         </is>
       </c>
-      <c r="H9" s="24" t="inlineStr">
+      <c r="H9" s="27" t="inlineStr">
         <is>
           <t>1. Em Dashboard, observar card Saldo Real
 2. Conferir que soma bate com total em Contas</t>
         </is>
       </c>
-      <c r="I9" s="24" t="inlineStr">
+      <c r="I9" s="27" t="inlineStr">
         <is>
           <t>Saldo agregado = soma dos saldos de contas com ativa=true</t>
         </is>
       </c>
-      <c r="J9" s="24" t="inlineStr">
+      <c r="J9" s="27" t="inlineStr">
         <is>
           <t>saldoRealPorConta.js + RF-068</t>
         </is>
       </c>
-      <c r="K9" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L9" s="24" t="n"/>
-      <c r="M9" s="24" t="n"/>
+      <c r="K9" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L9" s="27" t="n"/>
+      <c r="M9" s="27" t="n"/>
     </row>
     <row r="10" ht="45" customHeight="1" s="18">
       <c r="A10" s="26" t="n">
@@ -1485,63 +1535,63 @@
       <c r="M10" s="26" t="n"/>
     </row>
     <row r="11" ht="45.75" customHeight="1" s="18">
-      <c r="A11" s="24" t="n">
+      <c r="A11" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>TC-FLUXO-01</t>
         </is>
       </c>
-      <c r="C11" s="24" t="inlineStr">
+      <c r="C11" s="27" t="inlineStr">
         <is>
           <t>Futuro/FluxoCaixa</t>
         </is>
       </c>
-      <c r="D11" s="25" t="inlineStr">
+      <c r="D11" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E11" s="24" t="inlineStr">
+      <c r="E11" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F11" s="24" t="inlineStr">
+      <c r="F11" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G11" s="24" t="inlineStr">
+      <c r="G11" s="27" t="inlineStr">
         <is>
           <t>Compromissos — parcelas agregadas dos cartoes</t>
         </is>
       </c>
-      <c r="H11" s="24" t="inlineStr">
+      <c r="H11" s="27" t="inlineStr">
         <is>
           <t>1. Navbar Futuro &gt; Fluxo de Caixa
 2. Scroll ate secao Compromissos Comprometidos (6 meses)
 3. Verificar agrupamento por mesFatura</t>
         </is>
       </c>
-      <c r="I11" s="24" t="inlineStr">
+      <c r="I11" s="27" t="inlineStr">
         <is>
           <t>Projecoes de todos os cartoes aparecem agregadas por mes; valores batem com aba Projecoes de cada cartao em /fatura.html</t>
         </is>
       </c>
-      <c r="J11" s="24" t="inlineStr">
+      <c r="J11" s="27" t="inlineStr">
         <is>
           <t>projecoesCartao.buscarProjecoesAgregadas + RF-063</t>
         </is>
       </c>
-      <c r="K11" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L11" s="24" t="n"/>
-      <c r="M11" s="24" t="n"/>
+      <c r="K11" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L11" s="27" t="n"/>
+      <c r="M11" s="27" t="n"/>
     </row>
     <row r="12" ht="45.75" customHeight="1" s="18">
       <c r="A12" s="26" t="n">
@@ -1603,62 +1653,62 @@
       <c r="M12" s="26" t="n"/>
     </row>
     <row r="13" ht="45" customHeight="1" s="18">
-      <c r="A13" s="24" t="n">
+      <c r="A13" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>TC-FLUXO-03</t>
         </is>
       </c>
-      <c r="C13" s="24" t="inlineStr">
+      <c r="C13" s="27" t="inlineStr">
         <is>
           <t>Futuro/FluxoCaixa</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E13" s="24" t="inlineStr">
+      <c r="E13" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F13" s="24" t="inlineStr">
+      <c r="F13" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G13" s="24" t="inlineStr">
+      <c r="G13" s="27" t="inlineStr">
         <is>
           <t>Forecast 6 meses renderiza</t>
         </is>
       </c>
-      <c r="H13" s="24" t="inlineStr">
+      <c r="H13" s="27" t="inlineStr">
         <is>
           <t>1. Em Fluxo de Caixa, observar card Forecast
 2. Verificar 6 barras (mes atual + 5 futuros)</t>
         </is>
       </c>
-      <c r="I13" s="24" t="inlineStr">
+      <c r="I13" s="27" t="inlineStr">
         <is>
           <t>Grafico Chart.js renderiza; tooltips mostram valores; cores alinhadas ao DS; tipografia via tokens</t>
         </is>
       </c>
-      <c r="J13" s="24" t="inlineStr">
+      <c r="J13" s="27" t="inlineStr">
         <is>
           <t>forecastEngine.js + RF-067 + NRF-UX F7</t>
         </is>
       </c>
-      <c r="K13" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L13" s="24" t="n"/>
-      <c r="M13" s="24" t="n"/>
+      <c r="K13" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L13" s="27" t="n"/>
+      <c r="M13" s="27" t="n"/>
     </row>
     <row r="14" ht="45.75" customHeight="1" s="18">
       <c r="A14" s="26" t="n">
@@ -1720,61 +1770,61 @@
       <c r="M14" s="26" t="n"/>
     </row>
     <row r="15" ht="45" customHeight="1" s="18">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>TC-PAT-02</t>
         </is>
       </c>
-      <c r="C15" s="24" t="inlineStr">
+      <c r="C15" s="27" t="inlineStr">
         <is>
           <t>Historico/Patrimonio</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E15" s="24" t="inlineStr">
+      <c r="E15" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F15" s="24" t="inlineStr">
+      <c r="F15" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G15" s="24" t="inlineStr">
+      <c r="G15" s="27" t="inlineStr">
         <is>
           <t>Grafico de evolucao patrimonial renderiza</t>
         </is>
       </c>
-      <c r="H15" s="24" t="inlineStr">
+      <c r="H15" s="27" t="inlineStr">
         <is>
           <t>1. Em Patrimonio, observar grafico de evolucao mensal</t>
         </is>
       </c>
-      <c r="I15" s="24" t="inlineStr">
+      <c r="I15" s="27" t="inlineStr">
         <is>
           <t>Chart renderiza; sem NaN nas series; legenda usa tokens DS</t>
         </is>
       </c>
-      <c r="J15" s="24" t="inlineStr">
+      <c r="J15" s="27" t="inlineStr">
         <is>
           <t>RF-066 PR #178</t>
         </is>
       </c>
-      <c r="K15" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L15" s="24" t="n"/>
-      <c r="M15" s="24" t="n"/>
+      <c r="K15" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L15" s="27" t="n"/>
+      <c r="M15" s="27" t="n"/>
     </row>
     <row r="16" ht="45.75" customHeight="1" s="18">
       <c r="A16" s="26" t="n">
@@ -1790,7 +1840,7 @@
           <t>Transacoes/Despesas</t>
         </is>
       </c>
-      <c r="D16" s="25" t="inlineStr">
+      <c r="D16" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -1836,62 +1886,62 @@
       <c r="M16" s="26" t="n"/>
     </row>
     <row r="17" ht="45" customHeight="1" s="18">
-      <c r="A17" s="24" t="n">
+      <c r="A17" s="27" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>TC-DESP-02</t>
         </is>
       </c>
-      <c r="C17" s="24" t="inlineStr">
+      <c r="C17" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Despesas</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E17" s="24" t="inlineStr">
+      <c r="E17" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F17" s="24" t="inlineStr">
+      <c r="F17" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G17" s="24" t="inlineStr">
+      <c r="G17" s="27" t="inlineStr">
         <is>
           <t>Listagem usa progressive disclosure (ENH-004)</t>
         </is>
       </c>
-      <c r="H17" s="24" t="inlineStr">
+      <c r="H17" s="27" t="inlineStr">
         <is>
           <t>1. Em Despesas, observar linhas da listagem
 2. Identificar linha com multiplos metadados (ex: despesa conjunta parcelada)</t>
         </is>
       </c>
-      <c r="I17" s="24" t="inlineStr">
+      <c r="I17" s="27" t="inlineStr">
         <is>
           <t>Linha compacta mostra 1 badge (hierarquia: transferencia &gt; projecao &gt; parcela &gt; conjunta &gt; portador). Toggle &gt; aparece quando ha &gt;1 metadado</t>
         </is>
       </c>
-      <c r="J17" s="24" t="inlineStr">
+      <c r="J17" s="27" t="inlineStr">
         <is>
           <t>ENH-004 PR #185</t>
         </is>
       </c>
-      <c r="K17" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L17" s="24" t="n"/>
-      <c r="M17" s="24" t="n"/>
+      <c r="K17" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L17" s="27" t="n"/>
+      <c r="M17" s="27" t="n"/>
     </row>
     <row r="18" ht="45.75" customHeight="1" s="18">
       <c r="A18" s="26" t="n">
@@ -1953,63 +2003,63 @@
       <c r="M18" s="26" t="n"/>
     </row>
     <row r="19" ht="45.75" customHeight="1" s="18">
-      <c r="A19" s="24" t="n">
+      <c r="A19" s="27" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="24" t="inlineStr">
+      <c r="B19" s="27" t="inlineStr">
         <is>
           <t>TC-DESP-04</t>
         </is>
       </c>
-      <c r="C19" s="24" t="inlineStr">
+      <c r="C19" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Despesas</t>
         </is>
       </c>
-      <c r="D19" s="25" t="inlineStr">
+      <c r="D19" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E19" s="24" t="inlineStr">
+      <c r="E19" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F19" s="24" t="inlineStr">
+      <c r="F19" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G19" s="24" t="inlineStr">
+      <c r="G19" s="27" t="inlineStr">
         <is>
           <t>CRUD de despesa manual preserva mesFatura + chave_dedup</t>
         </is>
       </c>
-      <c r="H19" s="24" t="inlineStr">
+      <c r="H19" s="27" t="inlineStr">
         <is>
           <t>1. Criar despesa de cartao manual
 2. Abrir DevTools &gt; Firestore emulator ou inspecionar via database.js
 3. Verificar chave_dedup formato manual||... e mesFatura=YYYY-MM</t>
         </is>
       </c>
-      <c r="I19" s="24" t="inlineStr">
+      <c r="I19" s="27" t="inlineStr">
         <is>
           <t>Campos corretos; sem undefined; sem null onde deveria ter valor</t>
         </is>
       </c>
-      <c r="J19" s="24" t="inlineStr">
+      <c r="J19" s="27" t="inlineStr">
         <is>
           <t>CLAUDE.md - chave_dedup + mesFatura + BUG-021/022/026/032</t>
         </is>
       </c>
-      <c r="K19" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L19" s="24" t="n"/>
-      <c r="M19" s="24" t="n"/>
+      <c r="K19" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L19" s="27" t="n"/>
+      <c r="M19" s="27" t="n"/>
     </row>
     <row r="20" ht="45" customHeight="1" s="18">
       <c r="A20" s="26" t="n">
@@ -2070,63 +2120,63 @@
       <c r="M20" s="26" t="n"/>
     </row>
     <row r="21" ht="45.75" customHeight="1" s="18">
-      <c r="A21" s="24" t="n">
+      <c r="A21" s="27" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="24" t="inlineStr">
+      <c r="B21" s="27" t="inlineStr">
         <is>
           <t>TC-REC-02</t>
         </is>
       </c>
-      <c r="C21" s="24" t="inlineStr">
+      <c r="C21" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Receitas</t>
         </is>
       </c>
-      <c r="D21" s="24" t="inlineStr">
+      <c r="D21" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E21" s="24" t="inlineStr">
+      <c r="E21" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F21" s="24" t="inlineStr">
+      <c r="F21" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G21" s="24" t="inlineStr">
+      <c r="G21" s="27" t="inlineStr">
         <is>
           <t>Receita recorrente gera projecao futura</t>
         </is>
       </c>
-      <c r="H21" s="24" t="inlineStr">
+      <c r="H21" s="27" t="inlineStr">
         <is>
           <t>1. Criar receita com recorrencia mensal
 2. Abrir Fluxo de Caixa
 3. Observar se aparece nos proximos meses</t>
         </is>
       </c>
-      <c r="I21" s="24" t="inlineStr">
+      <c r="I21" s="27" t="inlineStr">
         <is>
           <t>Projecao aparece com tipo correto; nao duplica no mes de criacao</t>
         </is>
       </c>
-      <c r="J21" s="24" t="inlineStr">
+      <c r="J21" s="27" t="inlineStr">
         <is>
           <t>recurringDetector.js</t>
         </is>
       </c>
-      <c r="K21" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L21" s="24" t="n"/>
-      <c r="M21" s="24" t="n"/>
+      <c r="K21" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L21" s="27" t="n"/>
+      <c r="M21" s="27" t="n"/>
     </row>
     <row r="22" ht="45.75" customHeight="1" s="18">
       <c r="A22" s="26" t="n">
@@ -2188,63 +2238,63 @@
       <c r="M22" s="26" t="n"/>
     </row>
     <row r="23" ht="45.75" customHeight="1" s="18">
-      <c r="A23" s="24" t="n">
+      <c r="A23" s="27" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="24" t="inlineStr">
+      <c r="B23" s="27" t="inlineStr">
         <is>
           <t>TC-FAT-02</t>
         </is>
       </c>
-      <c r="C23" s="24" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Fatura</t>
         </is>
       </c>
-      <c r="D23" s="25" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E23" s="24" t="inlineStr">
+      <c r="E23" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F23" s="24" t="inlineStr">
+      <c r="F23" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G23" s="24" t="inlineStr">
+      <c r="G23" s="27" t="inlineStr">
         <is>
           <t>Reconciliacao fatura vs extrato (RF-062/063/064)</t>
         </is>
       </c>
-      <c r="H23" s="24" t="inlineStr">
+      <c r="H23" s="27" t="inlineStr">
         <is>
           <t>1. Importar fatura do cartao
 2. Abrir aba Reconciliacao
 3. Verificar match exato + fuzzy + ajustes marketplace</t>
         </is>
       </c>
-      <c r="I23" s="24" t="inlineStr">
+      <c r="I23" s="27" t="inlineStr">
         <is>
           <t>Matches exatos destacados; fuzzy com highlight amber; ajustes marketplace sugerem reconciliacao</t>
         </is>
       </c>
-      <c r="J23" s="24" t="inlineStr">
+      <c r="J23" s="27" t="inlineStr">
         <is>
           <t>reconciliadorFatura.js + ajusteDetector.js</t>
         </is>
       </c>
-      <c r="K23" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L23" s="24" t="n"/>
-      <c r="M23" s="24" t="n"/>
+      <c r="K23" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L23" s="27" t="n"/>
+      <c r="M23" s="27" t="n"/>
     </row>
     <row r="24" ht="45" customHeight="1" s="18">
       <c r="A24" s="26" t="n">
@@ -2305,63 +2355,63 @@
       <c r="M24" s="26" t="n"/>
     </row>
     <row r="25" ht="45.75" customHeight="1" s="18">
-      <c r="A25" s="24" t="n">
+      <c r="A25" s="27" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="24" t="inlineStr">
+      <c r="B25" s="27" t="inlineStr">
         <is>
           <t>TC-IMP-01</t>
         </is>
       </c>
-      <c r="C25" s="24" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Importar</t>
         </is>
       </c>
-      <c r="D25" s="25" t="inlineStr">
+      <c r="D25" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E25" s="24" t="inlineStr">
+      <c r="E25" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F25" s="24" t="inlineStr">
+      <c r="F25" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G25" s="24" t="inlineStr">
+      <c r="G25" s="27" t="inlineStr">
         <is>
           <t>Import CSV banco — dedup funciona</t>
         </is>
       </c>
-      <c r="H25" s="24" t="inlineStr">
+      <c r="H25" s="27" t="inlineStr">
         <is>
           <t>1. Navbar Transacoes &gt; Importar
 2. Upload CSV de banco conhecido (ex: Itau, Nubank)
 3. Re-upload do MESMO arquivo</t>
         </is>
       </c>
-      <c r="I25" s="24" t="inlineStr">
+      <c r="I25" s="27" t="inlineStr">
         <is>
           <t>Primeira importacao: linhas novas criadas com chave_dedup. Segunda: 0 linhas duplicadas criadas; dedup via buscarChavesDedup</t>
         </is>
       </c>
-      <c r="J25" s="24" t="inlineStr">
+      <c r="J25" s="27" t="inlineStr">
         <is>
           <t>deduplicador.js + chave_dedup (REGRA INVIOLAVEL 1)</t>
         </is>
       </c>
-      <c r="K25" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L25" s="24" t="n"/>
-      <c r="M25" s="24" t="n"/>
+      <c r="K25" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L25" s="27" t="n"/>
+      <c r="M25" s="27" t="n"/>
     </row>
     <row r="26" ht="45.75" customHeight="1" s="18">
       <c r="A26" s="26" t="n">
@@ -2377,7 +2427,7 @@
           <t>Transacoes/Importar</t>
         </is>
       </c>
-      <c r="D26" s="25" t="inlineStr">
+      <c r="D26" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -2423,62 +2473,62 @@
       <c r="M26" s="26" t="n"/>
     </row>
     <row r="27" ht="45" customHeight="1" s="18">
-      <c r="A27" s="24" t="n">
+      <c r="A27" s="27" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="24" t="inlineStr">
+      <c r="B27" s="27" t="inlineStr">
         <is>
           <t>TC-IMP-03</t>
         </is>
       </c>
-      <c r="C27" s="24" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Importar</t>
         </is>
       </c>
-      <c r="D27" s="24" t="inlineStr">
+      <c r="D27" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E27" s="24" t="inlineStr">
+      <c r="E27" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F27" s="24" t="inlineStr">
+      <c r="F27" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G27" s="24" t="inlineStr">
+      <c r="G27" s="27" t="inlineStr">
         <is>
           <t>Detector de transferencia interna</t>
         </is>
       </c>
-      <c r="H27" s="24" t="inlineStr">
+      <c r="H27" s="27" t="inlineStr">
         <is>
           <t>1. Importar extrato com TED entre contas Luigi e Ana
 2. Verificar que saida e entrada sao pareadas</t>
         </is>
       </c>
-      <c r="I27" s="24" t="inlineStr">
+      <c r="I27" s="27" t="inlineStr">
         <is>
           <t>tipo=transferencia_interna em ambos; nao infla despesas nem receitas do mes</t>
         </is>
       </c>
-      <c r="J27" s="24" t="inlineStr">
+      <c r="J27" s="27" t="inlineStr">
         <is>
           <t>detectorTransferenciaInterna.js</t>
         </is>
       </c>
-      <c r="K27" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L27" s="24" t="n"/>
-      <c r="M27" s="24" t="n"/>
+      <c r="K27" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L27" s="27" t="n"/>
+      <c r="M27" s="27" t="n"/>
     </row>
     <row r="28" ht="45" customHeight="1" s="18">
       <c r="A28" s="26" t="n">
@@ -2539,63 +2589,63 @@
       <c r="M28" s="26" t="n"/>
     </row>
     <row r="29" ht="45.75" customHeight="1" s="18">
-      <c r="A29" s="24" t="n">
+      <c r="A29" s="27" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="24" t="inlineStr">
+      <c r="B29" s="27" t="inlineStr">
         <is>
           <t>TC-CAT-01</t>
         </is>
       </c>
-      <c r="C29" s="24" t="inlineStr">
+      <c r="C29" s="27" t="inlineStr">
         <is>
           <t>Config/Categorias</t>
         </is>
       </c>
-      <c r="D29" s="24" t="inlineStr">
+      <c r="D29" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E29" s="24" t="inlineStr">
+      <c r="E29" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F29" s="24" t="inlineStr">
+      <c r="F29" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G29" s="24" t="inlineStr">
+      <c r="G29" s="27" t="inlineStr">
         <is>
           <t>Criar categoria com emoji e cor</t>
         </is>
       </c>
-      <c r="H29" s="24" t="inlineStr">
+      <c r="H29" s="27" t="inlineStr">
         <is>
           <t>1. Navbar Config &gt; Categorias
 2. Criar categoria com emoji + cor customizada
 3. Usar em nova despesa</t>
         </is>
       </c>
-      <c r="I29" s="24" t="inlineStr">
+      <c r="I29" s="27" t="inlineStr">
         <is>
           <t>Categoria aparece em listagens; cor reflete no badge; nao salva como sentinela __tipo__</t>
         </is>
       </c>
-      <c r="J29" s="24" t="inlineStr">
+      <c r="J29" s="27" t="inlineStr">
         <is>
           <t>CLAUDE.md + BUG-031 categoriaId sentinela</t>
         </is>
       </c>
-      <c r="K29" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L29" s="24" t="n"/>
-      <c r="M29" s="24" t="n"/>
+      <c r="K29" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L29" s="27" t="n"/>
+      <c r="M29" s="27" t="n"/>
     </row>
     <row r="30" ht="45" customHeight="1" s="18">
       <c r="A30" s="26" t="n">
@@ -2656,62 +2706,62 @@
       <c r="M30" s="26" t="n"/>
     </row>
     <row r="31" ht="45" customHeight="1" s="18">
-      <c r="A31" s="24" t="n">
+      <c r="A31" s="27" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="24" t="inlineStr">
+      <c r="B31" s="27" t="inlineStr">
         <is>
           <t>TC-ORC-01</t>
         </is>
       </c>
-      <c r="C31" s="24" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
         <is>
           <t>Config/Orcamentos</t>
         </is>
       </c>
-      <c r="D31" s="24" t="inlineStr">
+      <c r="D31" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E31" s="24" t="inlineStr">
+      <c r="E31" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F31" s="24" t="inlineStr">
+      <c r="F31" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G31" s="24" t="inlineStr">
+      <c r="G31" s="27" t="inlineStr">
         <is>
           <t>Cores de orcamento por faixa de %</t>
         </is>
       </c>
-      <c r="H31" s="24" t="inlineStr">
+      <c r="H31" s="27" t="inlineStr">
         <is>
           <t>1. Config &gt; Orcamentos
 2. Observar orcamentos em &lt; 70%, 70-89%, 90-100%, &gt; 100%</t>
         </is>
       </c>
-      <c r="I31" s="24" t="inlineStr">
+      <c r="I31" s="27" t="inlineStr">
         <is>
           <t>Cores: OK (verde) &lt;70%, Warning (amarelo) 70-89%, Danger (vermelho) 90-100%, Critical (roxo) &gt;100%</t>
         </is>
       </c>
-      <c r="J31" s="24" t="inlineStr">
+      <c r="J31" s="27" t="inlineStr">
         <is>
           <t>DESIGN_SYSTEM.md status orcamentos</t>
         </is>
       </c>
-      <c r="K31" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L31" s="24" t="n"/>
-      <c r="M31" s="24" t="n"/>
+      <c r="K31" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L31" s="27" t="n"/>
+      <c r="M31" s="27" t="n"/>
     </row>
     <row r="32" ht="45.75" customHeight="1" s="18">
       <c r="A32" s="26" t="n">
@@ -2727,7 +2777,7 @@
           <t>Config/Grupo</t>
         </is>
       </c>
-      <c r="D32" s="25" t="inlineStr">
+      <c r="D32" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -2773,63 +2823,63 @@
       <c r="M32" s="26" t="n"/>
     </row>
     <row r="33" ht="45.75" customHeight="1" s="18">
-      <c r="A33" s="24" t="n">
+      <c r="A33" s="27" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="24" t="inlineStr">
+      <c r="B33" s="27" t="inlineStr">
         <is>
           <t>TC-GRUPO-02</t>
         </is>
       </c>
-      <c r="C33" s="24" t="inlineStr">
+      <c r="C33" s="27" t="inlineStr">
         <is>
           <t>Config/Grupo</t>
         </is>
       </c>
-      <c r="D33" s="24" t="inlineStr">
+      <c r="D33" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E33" s="24" t="inlineStr">
+      <c r="E33" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F33" s="24" t="inlineStr">
+      <c r="F33" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G33" s="24" t="inlineStr">
+      <c r="G33" s="27" t="inlineStr">
         <is>
           <t>Convite de membro via email</t>
         </is>
       </c>
-      <c r="H33" s="24" t="inlineStr">
+      <c r="H33" s="27" t="inlineStr">
         <is>
           <t>1. Config &gt; Grupo
 2. Enviar convite para email de teste
 3. Aceitar convite em outra sessao</t>
         </is>
       </c>
-      <c r="I33" s="24" t="inlineStr">
+      <c r="I33" s="27" t="inlineStr">
         <is>
           <t>Novo membro entra no grupo; acesso compartilhado funciona</t>
         </is>
       </c>
-      <c r="J33" s="24" t="inlineStr">
+      <c r="J33" s="27" t="inlineStr">
         <is>
           <t>src/js/services/grupos.js</t>
         </is>
       </c>
-      <c r="K33" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L33" s="24" t="n"/>
-      <c r="M33" s="24" t="n"/>
+      <c r="K33" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L33" s="27" t="n"/>
+      <c r="M33" s="27" t="n"/>
     </row>
     <row r="34" ht="60" customHeight="1" s="18">
       <c r="A34" s="26" t="n">
@@ -2892,63 +2942,63 @@
       <c r="M34" s="26" t="n"/>
     </row>
     <row r="35" ht="45.75" customHeight="1" s="18">
-      <c r="A35" s="24" t="n">
+      <c r="A35" s="27" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="24" t="inlineStr">
+      <c r="B35" s="27" t="inlineStr">
         <is>
           <t>TC-DS-02</t>
         </is>
       </c>
-      <c r="C35" s="24" t="inlineStr">
+      <c r="C35" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D35" s="24" t="inlineStr">
+      <c r="D35" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E35" s="24" t="inlineStr">
+      <c r="E35" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F35" s="24" t="inlineStr">
+      <c r="F35" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G35" s="24" t="inlineStr">
+      <c r="G35" s="27" t="inlineStr">
         <is>
           <t>.btn-danger:hover usa --shadow-danger</t>
         </is>
       </c>
-      <c r="H35" s="24" t="inlineStr">
+      <c r="H35" s="27" t="inlineStr">
         <is>
           <t>1. Abrir components.css
 2. Localizar .btn-danger:hover
 3. Verificar que shadow usa var(--shadow-danger)</t>
         </is>
       </c>
-      <c r="I35" s="24" t="inlineStr">
+      <c r="I35" s="27" t="inlineStr">
         <is>
           <t>Shadow aponta para token novo do Warm Finance; sem rgba hardcoded pre-rebrand</t>
         </is>
       </c>
-      <c r="J35" s="24" t="inlineStr">
+      <c r="J35" s="27" t="inlineStr">
         <is>
           <t>PR #190 CHANGELOG v3.38.0</t>
         </is>
       </c>
-      <c r="K35" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L35" s="24" t="n"/>
-      <c r="M35" s="24" t="n"/>
+      <c r="K35" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L35" s="27" t="n"/>
+      <c r="M35" s="27" t="n"/>
     </row>
     <row r="36" ht="45.75" customHeight="1" s="18">
       <c r="A36" s="26" t="n">
@@ -2964,7 +3014,7 @@
           <t>Seguranca</t>
         </is>
       </c>
-      <c r="D36" s="25" t="inlineStr">
+      <c r="D36" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -3010,63 +3060,63 @@
       <c r="M36" s="26" t="n"/>
     </row>
     <row r="37" ht="45.75" customHeight="1" s="18">
-      <c r="A37" s="24" t="n">
+      <c r="A37" s="27" t="n">
         <v>35</v>
       </c>
-      <c r="B37" s="24" t="inlineStr">
+      <c r="B37" s="27" t="inlineStr">
         <is>
           <t>TC-REG-01</t>
         </is>
       </c>
-      <c r="C37" s="24" t="inlineStr">
+      <c r="C37" s="27" t="inlineStr">
         <is>
           <t>Regressao/Inviolaveis</t>
         </is>
       </c>
-      <c r="D37" s="25" t="inlineStr">
+      <c r="D37" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E37" s="24" t="inlineStr">
+      <c r="E37" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F37" s="24" t="inlineStr">
+      <c r="F37" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G37" s="24" t="inlineStr">
+      <c r="G37" s="27" t="inlineStr">
         <is>
           <t>chave_dedup mantem formato original</t>
         </is>
       </c>
-      <c r="H37" s="24" t="inlineStr">
+      <c r="H37" s="27" t="inlineStr">
         <is>
           <t>1. Importar transacao
 2. Inspecionar doc no Firestore
 3. Conferir formato: data||desc||valor||portador||parcela</t>
         </is>
       </c>
-      <c r="I37" s="24" t="inlineStr">
+      <c r="I37" s="27" t="inlineStr">
         <is>
           <t>Formato identico ao documentado em CLAUDE.md; sem quebra historica de dedup</t>
         </is>
       </c>
-      <c r="J37" s="24" t="inlineStr">
+      <c r="J37" s="27" t="inlineStr">
         <is>
           <t>REGRA INVIOLAVEL 1</t>
         </is>
       </c>
-      <c r="K37" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L37" s="24" t="n"/>
-      <c r="M37" s="24" t="n"/>
+      <c r="K37" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L37" s="27" t="n"/>
+      <c r="M37" s="27" t="n"/>
     </row>
     <row r="38" ht="45" customHeight="1" s="18">
       <c r="A38" s="26" t="n">
@@ -3082,7 +3132,7 @@
           <t>Regressao/Inviolaveis</t>
         </is>
       </c>
-      <c r="D38" s="25" t="inlineStr">
+      <c r="D38" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -3127,62 +3177,62 @@
       <c r="M38" s="26" t="n"/>
     </row>
     <row r="39" ht="45" customHeight="1" s="18">
-      <c r="A39" s="24" t="n">
+      <c r="A39" s="27" t="n">
         <v>37</v>
       </c>
-      <c r="B39" s="24" t="inlineStr">
+      <c r="B39" s="27" t="inlineStr">
         <is>
           <t>TC-REG-03</t>
         </is>
       </c>
-      <c r="C39" s="24" t="inlineStr">
+      <c r="C39" s="27" t="inlineStr">
         <is>
           <t>Regressao/Inviolaveis</t>
         </is>
       </c>
-      <c r="D39" s="24" t="inlineStr">
+      <c r="D39" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E39" s="24" t="inlineStr">
+      <c r="E39" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F39" s="24" t="inlineStr">
+      <c r="F39" s="27" t="inlineStr">
         <is>
           <t>v3.38.0</t>
         </is>
       </c>
-      <c r="G39" s="24" t="inlineStr">
+      <c r="G39" s="27" t="inlineStr">
         <is>
           <t>Delete em lote usa writeBatch</t>
         </is>
       </c>
-      <c r="H39" s="24" t="inlineStr">
+      <c r="H39" s="27" t="inlineStr">
         <is>
           <t>1. Executar operacao de purge/limpeza em lote (emulador recomendado)
 2. Observar firestore.rules + codigo</t>
         </is>
       </c>
-      <c r="I39" s="24" t="inlineStr">
+      <c r="I39" s="27" t="inlineStr">
         <is>
           <t>Operacoes em lote envolvem writeBatch; sem deleteDoc iterativo solto</t>
         </is>
       </c>
-      <c r="J39" s="24" t="inlineStr">
+      <c r="J39" s="27" t="inlineStr">
         <is>
           <t>REGRA INVIOLAVEL 9</t>
         </is>
       </c>
-      <c r="K39" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L39" s="24" t="n"/>
-      <c r="M39" s="24" t="n"/>
+      <c r="K39" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L39" s="27" t="n"/>
+      <c r="M39" s="27" t="n"/>
     </row>
     <row r="40" ht="45" customHeight="1" s="18">
       <c r="A40" s="26" t="n">
@@ -3243,40 +3293,40 @@
       <c r="M40" s="26" t="n"/>
     </row>
     <row r="41" ht="60" customHeight="1" s="18">
-      <c r="A41" s="24" t="n">
+      <c r="A41" s="27" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="24" t="inlineStr">
+      <c r="B41" s="27" t="inlineStr">
         <is>
           <t>TC-HERO-02</t>
         </is>
       </c>
-      <c r="C41" s="24" t="inlineStr">
+      <c r="C41" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Dashboard</t>
         </is>
       </c>
-      <c r="D41" s="24" t="inlineStr">
+      <c r="D41" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E41" s="24" t="inlineStr">
+      <c r="E41" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F41" s="24" t="inlineStr">
+      <c r="F41" s="27" t="inlineStr">
         <is>
           <t>v3.39.0</t>
         </is>
       </c>
-      <c r="G41" s="24" t="inlineStr">
+      <c r="G41" s="27" t="inlineStr">
         <is>
           <t>Card hero 'Proxima Fatura' condicional (&lt;=7 dias)</t>
         </is>
       </c>
-      <c r="H41" s="24" t="inlineStr">
+      <c r="H41" s="27" t="inlineStr">
         <is>
           <t>1. Garantir fatura com vencimento &lt;=7 dias
 2. Abrir dashboard
@@ -3284,23 +3334,23 @@
 4. Repetir com vencimento &gt;7 dias e verificar que some</t>
         </is>
       </c>
-      <c r="I41" s="24" t="inlineStr">
+      <c r="I41" s="27" t="inlineStr">
         <is>
           <t>Com &lt;=7 dias: card hero presente. Com &gt;7 dias: card some ou vira regular</t>
         </is>
       </c>
-      <c r="J41" s="24" t="inlineStr">
+      <c r="J41" s="27" t="inlineStr">
         <is>
           <t>NRF-VISUAL F1 + app.js regra condicional</t>
         </is>
       </c>
-      <c r="K41" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L41" s="24" t="n"/>
-      <c r="M41" s="24" t="n"/>
+      <c r="K41" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L41" s="27" t="n"/>
+      <c r="M41" s="27" t="n"/>
     </row>
     <row r="42" ht="60" customHeight="1" s="18">
       <c r="A42" s="26" t="n">
@@ -3363,62 +3413,62 @@
       <c r="M42" s="26" t="n"/>
     </row>
     <row r="43" ht="45" customHeight="1" s="18">
-      <c r="A43" s="24" t="n">
+      <c r="A43" s="27" t="n">
         <v>41</v>
       </c>
-      <c r="B43" s="24" t="inlineStr">
+      <c r="B43" s="27" t="inlineStr">
         <is>
           <t>TC-HERO-04</t>
         </is>
       </c>
-      <c r="C43" s="24" t="inlineStr">
+      <c r="C43" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Dashboard</t>
         </is>
       </c>
-      <c r="D43" s="24" t="inlineStr">
+      <c r="D43" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E43" s="24" t="inlineStr">
+      <c r="E43" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F43" s="24" t="inlineStr">
+      <c r="F43" s="27" t="inlineStr">
         <is>
           <t>v3.39.0</t>
         </is>
       </c>
-      <c r="G43" s="24" t="inlineStr">
+      <c r="G43" s="27" t="inlineStr">
         <is>
           <t>Contraste visual cards hero &gt;= 12:1</t>
         </is>
       </c>
-      <c r="H43" s="24" t="inlineStr">
+      <c r="H43" s="27" t="inlineStr">
         <is>
           <t>1. Em dashboard, abrir DevTools &gt; Lighthouse ou axe
 2. Rodar audit a11y nos cards hero</t>
         </is>
       </c>
-      <c r="I43" s="24" t="inlineStr">
+      <c r="I43" s="27" t="inlineStr">
         <is>
           <t>Contraste texto/fundo &gt;= 12:1 (AAA); sem warning a11y para cards hero</t>
         </is>
       </c>
-      <c r="J43" s="24" t="inlineStr">
+      <c r="J43" s="27" t="inlineStr">
         <is>
           <t>NRF-VISUAL F1 + DESIGN_SYSTEM.md contraste</t>
         </is>
       </c>
-      <c r="K43" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L43" s="24" t="n"/>
-      <c r="M43" s="24" t="n"/>
+      <c r="K43" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L43" s="27" t="n"/>
+      <c r="M43" s="27" t="n"/>
     </row>
     <row r="44" ht="45" customHeight="1" s="18">
       <c r="A44" s="26" t="n">
@@ -3479,63 +3529,63 @@
       <c r="M44" s="26" t="n"/>
     </row>
     <row r="45" ht="45.75" customHeight="1" s="18">
-      <c r="A45" s="24" t="n">
+      <c r="A45" s="27" t="n">
         <v>43</v>
       </c>
-      <c r="B45" s="24" t="inlineStr">
+      <c r="B45" s="27" t="inlineStr">
         <is>
           <t>TC-TYPO-01</t>
         </is>
       </c>
-      <c r="C45" s="24" t="inlineStr">
+      <c r="C45" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D45" s="24" t="inlineStr">
+      <c r="D45" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E45" s="24" t="inlineStr">
+      <c r="E45" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F45" s="24" t="inlineStr">
+      <c r="F45" s="27" t="inlineStr">
         <is>
           <t>v3.39.1</t>
         </is>
       </c>
-      <c r="G45" s="24" t="inlineStr">
+      <c r="G45" s="27" t="inlineStr">
         <is>
           <t>Fraunces carrega em titulos h1/h2 com fallback</t>
         </is>
       </c>
-      <c r="H45" s="24" t="inlineStr">
+      <c r="H45" s="27" t="inlineStr">
         <is>
           <t>1. Abrir qualquer pagina (dashboard, fatura)
 2. Inspecionar h1/h2 no DevTools &gt; Computed &gt; font-family
 3. Desabilitar cache e recarregar</t>
         </is>
       </c>
-      <c r="I45" s="24" t="inlineStr">
+      <c r="I45" s="27" t="inlineStr">
         <is>
           <t>font-family inclui Fraunces como primaria e fallback serif/system; renderizacao consistente</t>
         </is>
       </c>
-      <c r="J45" s="24" t="inlineStr">
+      <c r="J45" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F2 PR #194 + components.css</t>
         </is>
       </c>
-      <c r="K45" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L45" s="24" t="n"/>
-      <c r="M45" s="24" t="n"/>
+      <c r="K45" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L45" s="27" t="n"/>
+      <c r="M45" s="27" t="n"/>
     </row>
     <row r="46" ht="45.75" customHeight="1" s="18">
       <c r="A46" s="26" t="n">
@@ -3597,63 +3647,63 @@
       <c r="M46" s="26" t="n"/>
     </row>
     <row r="47" ht="45.75" customHeight="1" s="18">
-      <c r="A47" s="24" t="n">
+      <c r="A47" s="27" t="n">
         <v>45</v>
       </c>
-      <c r="B47" s="24" t="inlineStr">
+      <c r="B47" s="27" t="inlineStr">
         <is>
           <t>TC-ICON-01</t>
         </is>
       </c>
-      <c r="C47" s="24" t="inlineStr">
+      <c r="C47" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D47" s="25" t="inlineStr">
+      <c r="D47" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E47" s="24" t="inlineStr">
+      <c r="E47" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F47" s="24" t="inlineStr">
+      <c r="F47" s="27" t="inlineStr">
         <is>
           <t>v3.39.2</t>
         </is>
       </c>
-      <c r="G47" s="24" t="inlineStr">
+      <c r="G47" s="27" t="inlineStr">
         <is>
           <t>Navbar — 15 icones Lucide renderizam em todas as paginas</t>
         </is>
       </c>
-      <c r="H47" s="24" t="inlineStr">
+      <c r="H47" s="27" t="inlineStr">
         <is>
           <t>1. Visitar as 13 paginas do MPA
 2. Observar navbar em cada uma
 3. Verificar que icones das secoes Cockpit/Historico/Transacoes/Futuro/Config aparecem</t>
         </is>
       </c>
-      <c r="I47" s="24" t="inlineStr">
+      <c r="I47" s="27" t="inlineStr">
         <is>
           <t>Todos os 15 icones Lucide visiveis; zero quebra; sem rectangulos tofu</t>
         </is>
       </c>
-      <c r="J47" s="24" t="inlineStr">
+      <c r="J47" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F3 PR #195 + nav.js</t>
         </is>
       </c>
-      <c r="K47" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L47" s="24" t="n"/>
-      <c r="M47" s="24" t="n"/>
+      <c r="K47" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L47" s="27" t="n"/>
+      <c r="M47" s="27" t="n"/>
     </row>
     <row r="48" ht="45" customHeight="1" s="18">
       <c r="A48" s="26" t="n">
@@ -3669,7 +3719,7 @@
           <t>Design System</t>
         </is>
       </c>
-      <c r="D48" s="25" t="inlineStr">
+      <c r="D48" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -3714,62 +3764,62 @@
       <c r="M48" s="26" t="n"/>
     </row>
     <row r="49" ht="45" customHeight="1" s="18">
-      <c r="A49" s="24" t="n">
+      <c r="A49" s="27" t="n">
         <v>47</v>
       </c>
-      <c r="B49" s="24" t="inlineStr">
+      <c r="B49" s="27" t="inlineStr">
         <is>
           <t>TC-ICON-03</t>
         </is>
       </c>
-      <c r="C49" s="24" t="inlineStr">
+      <c r="C49" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D49" s="24" t="inlineStr">
+      <c r="D49" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E49" s="24" t="inlineStr">
+      <c r="E49" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F49" s="24" t="inlineStr">
+      <c r="F49" s="27" t="inlineStr">
         <is>
           <t>v3.39.3</t>
         </is>
       </c>
-      <c r="G49" s="24" t="inlineStr">
+      <c r="G49" s="27" t="inlineStr">
         <is>
           <t>Botoes canonicos usam icones Lucide</t>
         </is>
       </c>
-      <c r="H49" s="24" t="inlineStr">
+      <c r="H49" s="27" t="inlineStr">
         <is>
           <t>1. Observar botoes editar/excluir/salvar/fechar em despesas, receitas, contas
 2. Inspecionar HTML</t>
         </is>
       </c>
-      <c r="I49" s="24" t="inlineStr">
+      <c r="I49" s="27" t="inlineStr">
         <is>
           <t>Botoes usam &lt;i data-lucide='pencil|trash|save|x'&gt; com tokens --icon-size-*</t>
         </is>
       </c>
-      <c r="J49" s="24" t="inlineStr">
+      <c r="J49" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F4 PR #196</t>
         </is>
       </c>
-      <c r="K49" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L49" s="24" t="n"/>
-      <c r="M49" s="24" t="n"/>
+      <c r="K49" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L49" s="27" t="n"/>
+      <c r="M49" s="27" t="n"/>
     </row>
     <row r="50" ht="45.75" customHeight="1" s="18">
       <c r="A50" s="26" t="n">
@@ -3785,7 +3835,7 @@
           <t>Design System</t>
         </is>
       </c>
-      <c r="D50" s="25" t="inlineStr">
+      <c r="D50" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -3831,63 +3881,63 @@
       <c r="M50" s="26" t="n"/>
     </row>
     <row r="51" ht="45.75" customHeight="1" s="18">
-      <c r="A51" s="24" t="n">
+      <c r="A51" s="27" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="24" t="inlineStr">
+      <c r="B51" s="27" t="inlineStr">
         <is>
           <t>TC-ICON-05</t>
         </is>
       </c>
-      <c r="C51" s="24" t="inlineStr">
+      <c r="C51" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D51" s="25" t="inlineStr">
+      <c r="D51" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E51" s="24" t="inlineStr">
+      <c r="E51" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F51" s="24" t="inlineStr">
+      <c r="F51" s="27" t="inlineStr">
         <is>
           <t>v3.39.2</t>
         </is>
       </c>
-      <c r="G51" s="24" t="inlineStr">
+      <c r="G51" s="27" t="inlineStr">
         <is>
           <t>Zero emojis em chrome (navbar, headers, botoes)</t>
         </is>
       </c>
-      <c r="H51" s="24" t="inlineStr">
+      <c r="H51" s="27" t="inlineStr">
         <is>
           <t>1. Abrir DevTools &gt; Console
 2. Rodar: document.body.innerText.match(/[\u{1F300}-\u{1F9FF}]/gu)?.length
 3. Verificar resultado</t>
         </is>
       </c>
-      <c r="I51" s="24" t="inlineStr">
+      <c r="I51" s="27" t="inlineStr">
         <is>
           <t>Contagem de emojis em chrome = 0 (categorias de usuario podem ter emojis, mas UI nao)</t>
         </is>
       </c>
-      <c r="J51" s="24" t="inlineStr">
+      <c r="J51" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F3 + grep emoji removal</t>
         </is>
       </c>
-      <c r="K51" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L51" s="24" t="n"/>
-      <c r="M51" s="24" t="n"/>
+      <c r="K51" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L51" s="27" t="n"/>
+      <c r="M51" s="27" t="n"/>
     </row>
     <row r="52" ht="45.75" customHeight="1" s="18">
       <c r="A52" s="26" t="n">
@@ -3949,62 +3999,62 @@
       <c r="M52" s="26" t="n"/>
     </row>
     <row r="53" ht="45" customHeight="1" s="18">
-      <c r="A53" s="24" t="n">
+      <c r="A53" s="27" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="24" t="inlineStr">
+      <c r="B53" s="27" t="inlineStr">
         <is>
           <t>TC-SKEL-01</t>
         </is>
       </c>
-      <c r="C53" s="24" t="inlineStr">
+      <c r="C53" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Dashboard</t>
         </is>
       </c>
-      <c r="D53" s="25" t="inlineStr">
+      <c r="D53" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E53" s="24" t="inlineStr">
+      <c r="E53" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F53" s="24" t="inlineStr">
+      <c r="F53" s="27" t="inlineStr">
         <is>
           <t>v3.39.4</t>
         </is>
       </c>
-      <c r="G53" s="24" t="inlineStr">
+      <c r="G53" s="27" t="inlineStr">
         <is>
           <t>Dashboard — skeleton visivel antes de onSnapshot</t>
         </is>
       </c>
-      <c r="H53" s="24" t="inlineStr">
+      <c r="H53" s="27" t="inlineStr">
         <is>
           <t>1. Abrir /dashboard.html com DevTools &gt; Network &gt; Slow 3G
 2. Observar estado inicial pre-dados</t>
         </is>
       </c>
-      <c r="I53" s="24" t="inlineStr">
+      <c r="I53" s="27" t="inlineStr">
         <is>
           <t>Skeleton shimmer aparece nos cards; canvas Chart.js oculto; desaparece ao render real</t>
         </is>
       </c>
-      <c r="J53" s="24" t="inlineStr">
+      <c r="J53" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F5 PR #197 + skeletons.js</t>
         </is>
       </c>
-      <c r="K53" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L53" s="24" t="n"/>
-      <c r="M53" s="24" t="n"/>
+      <c r="K53" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L53" s="27" t="n"/>
+      <c r="M53" s="27" t="n"/>
     </row>
     <row r="54" ht="45.75" customHeight="1" s="18">
       <c r="A54" s="26" t="n">
@@ -4020,7 +4070,7 @@
           <t>Transacoes/Fatura</t>
         </is>
       </c>
-      <c r="D54" s="25" t="inlineStr">
+      <c r="D54" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -4066,62 +4116,62 @@
       <c r="M54" s="26" t="n"/>
     </row>
     <row r="55" ht="45" customHeight="1" s="18">
-      <c r="A55" s="24" t="n">
+      <c r="A55" s="27" t="n">
         <v>53</v>
       </c>
-      <c r="B55" s="24" t="inlineStr">
+      <c r="B55" s="27" t="inlineStr">
         <is>
           <t>TC-SKEL-03</t>
         </is>
       </c>
-      <c r="C55" s="24" t="inlineStr">
+      <c r="C55" s="27" t="inlineStr">
         <is>
           <t>Historico/Patrimonio</t>
         </is>
       </c>
-      <c r="D55" s="24" t="inlineStr">
+      <c r="D55" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E55" s="24" t="inlineStr">
+      <c r="E55" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F55" s="24" t="inlineStr">
+      <c r="F55" s="27" t="inlineStr">
         <is>
           <t>v3.39.4</t>
         </is>
       </c>
-      <c r="G55" s="24" t="inlineStr">
+      <c r="G55" s="27" t="inlineStr">
         <is>
           <t>Patrimonio — skeleton de ativos e passivos</t>
         </is>
       </c>
-      <c r="H55" s="24" t="inlineStr">
+      <c r="H55" s="27" t="inlineStr">
         <is>
           <t>1. Navbar Historico &gt; Patrimonio (cold load)
 2. Observar cards de ativos e passivos antes da hidratacao</t>
         </is>
       </c>
-      <c r="I55" s="24" t="inlineStr">
+      <c r="I55" s="27" t="inlineStr">
         <is>
           <t>Skeleton dos cards aparece; substituido pelos valores reais</t>
         </is>
       </c>
-      <c r="J55" s="24" t="inlineStr">
+      <c r="J55" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F5 + patrimonio.js</t>
         </is>
       </c>
-      <c r="K55" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L55" s="24" t="n"/>
-      <c r="M55" s="24" t="n"/>
+      <c r="K55" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L55" s="27" t="n"/>
+      <c r="M55" s="27" t="n"/>
     </row>
     <row r="56" ht="45" customHeight="1" s="18">
       <c r="A56" s="26" t="n">
@@ -4182,62 +4232,62 @@
       <c r="M56" s="26" t="n"/>
     </row>
     <row r="57" ht="45" customHeight="1" s="18">
-      <c r="A57" s="24" t="n">
+      <c r="A57" s="27" t="n">
         <v>55</v>
       </c>
-      <c r="B57" s="24" t="inlineStr">
+      <c r="B57" s="27" t="inlineStr">
         <is>
           <t>TC-SKEL-05</t>
         </is>
       </c>
-      <c r="C57" s="24" t="inlineStr">
+      <c r="C57" s="27" t="inlineStr">
         <is>
           <t>Futuro/FluxoCaixa</t>
         </is>
       </c>
-      <c r="D57" s="24" t="inlineStr">
+      <c r="D57" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E57" s="24" t="inlineStr">
+      <c r="E57" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F57" s="24" t="inlineStr">
+      <c r="F57" s="27" t="inlineStr">
         <is>
           <t>v3.39.4</t>
         </is>
       </c>
-      <c r="G57" s="24" t="inlineStr">
+      <c r="G57" s="27" t="inlineStr">
         <is>
           <t>Fluxo de Caixa — skeleton de compromissos</t>
         </is>
       </c>
-      <c r="H57" s="24" t="inlineStr">
+      <c r="H57" s="27" t="inlineStr">
         <is>
           <t>1. Em Fluxo de Caixa, scroll ate Compromissos (cold load)
 2. Observar estado pre-render</t>
         </is>
       </c>
-      <c r="I57" s="24" t="inlineStr">
+      <c r="I57" s="27" t="inlineStr">
         <is>
           <t>Skeleton das linhas de compromissos aparece; trocas suave pelos dados reais</t>
         </is>
       </c>
-      <c r="J57" s="24" t="inlineStr">
+      <c r="J57" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F5</t>
         </is>
       </c>
-      <c r="K57" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L57" s="24" t="n"/>
-      <c r="M57" s="24" t="n"/>
+      <c r="K57" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L57" s="27" t="n"/>
+      <c r="M57" s="27" t="n"/>
     </row>
     <row r="58" ht="45" customHeight="1" s="18">
       <c r="A58" s="26" t="n">
@@ -4298,62 +4348,62 @@
       <c r="M58" s="26" t="n"/>
     </row>
     <row r="59" ht="45" customHeight="1" s="18">
-      <c r="A59" s="24" t="n">
+      <c r="A59" s="27" t="n">
         <v>57</v>
       </c>
-      <c r="B59" s="24" t="inlineStr">
+      <c r="B59" s="27" t="inlineStr">
         <is>
           <t>TC-SKEL-07</t>
         </is>
       </c>
-      <c r="C59" s="24" t="inlineStr">
+      <c r="C59" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D59" s="24" t="inlineStr">
+      <c r="D59" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E59" s="24" t="inlineStr">
+      <c r="E59" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F59" s="24" t="inlineStr">
+      <c r="F59" s="27" t="inlineStr">
         <is>
           <t>v3.39.4</t>
         </is>
       </c>
-      <c r="G59" s="24" t="inlineStr">
+      <c r="G59" s="27" t="inlineStr">
         <is>
           <t>Skeleton removido ao render — sem flash de conteudo antigo</t>
         </is>
       </c>
-      <c r="H59" s="24" t="inlineStr">
+      <c r="H59" s="27" t="inlineStr">
         <is>
           <t>1. Visitar dashboard, sair, voltar (simulando cache hit)
 2. Observar transicao</t>
         </is>
       </c>
-      <c r="I59" s="24" t="inlineStr">
+      <c r="I59" s="27" t="inlineStr">
         <is>
           <t>Sem flash do estado anterior; skeleton &gt;&gt; conteudo novo sem FOUC</t>
         </is>
       </c>
-      <c r="J59" s="24" t="inlineStr">
+      <c r="J59" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F5</t>
         </is>
       </c>
-      <c r="K59" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L59" s="24" t="n"/>
-      <c r="M59" s="24" t="n"/>
+      <c r="K59" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L59" s="27" t="n"/>
+      <c r="M59" s="27" t="n"/>
     </row>
     <row r="60" ht="45.75" customHeight="1" s="18">
       <c r="A60" s="26" t="n">
@@ -4415,62 +4465,62 @@
       <c r="M60" s="26" t="n"/>
     </row>
     <row r="61" ht="45" customHeight="1" s="18">
-      <c r="A61" s="24" t="n">
+      <c r="A61" s="27" t="n">
         <v>59</v>
       </c>
-      <c r="B61" s="24" t="inlineStr">
+      <c r="B61" s="27" t="inlineStr">
         <is>
           <t>TC-SKEL-09</t>
         </is>
       </c>
-      <c r="C61" s="24" t="inlineStr">
+      <c r="C61" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D61" s="24" t="inlineStr">
+      <c r="D61" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E61" s="24" t="inlineStr">
+      <c r="E61" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F61" s="24" t="inlineStr">
+      <c r="F61" s="27" t="inlineStr">
         <is>
           <t>v3.39.4</t>
         </is>
       </c>
-      <c r="G61" s="24" t="inlineStr">
+      <c r="G61" s="27" t="inlineStr">
         <is>
           <t>Skeleton ARIA — leitores de tela nao leem como conteudo</t>
         </is>
       </c>
-      <c r="H61" s="24" t="inlineStr">
+      <c r="H61" s="27" t="inlineStr">
         <is>
           <t>1. Inspecionar skeleton elements
 2. Verificar atributos aria-hidden ou role</t>
         </is>
       </c>
-      <c r="I61" s="24" t="inlineStr">
+      <c r="I61" s="27" t="inlineStr">
         <is>
           <t>Skeletons tem aria-hidden='true' ou role='presentation'; leitores ignoram</t>
         </is>
       </c>
-      <c r="J61" s="24" t="inlineStr">
+      <c r="J61" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F5 + acessibilidade</t>
         </is>
       </c>
-      <c r="K61" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L61" s="24" t="n"/>
-      <c r="M61" s="24" t="n"/>
+      <c r="K61" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L61" s="27" t="n"/>
+      <c r="M61" s="27" t="n"/>
     </row>
     <row r="62" ht="45.75" customHeight="1" s="18">
       <c r="A62" s="26" t="n">
@@ -4532,63 +4582,63 @@
       <c r="M62" s="26" t="n"/>
     </row>
     <row r="63" ht="45.75" customHeight="1" s="18">
-      <c r="A63" s="24" t="n">
+      <c r="A63" s="27" t="n">
         <v>61</v>
       </c>
-      <c r="B63" s="24" t="inlineStr">
+      <c r="B63" s="27" t="inlineStr">
         <is>
           <t>TC-SPC-02</t>
         </is>
       </c>
-      <c r="C63" s="24" t="inlineStr">
+      <c r="C63" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D63" s="24" t="inlineStr">
+      <c r="D63" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E63" s="24" t="inlineStr">
+      <c r="E63" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F63" s="24" t="inlineStr">
+      <c r="F63" s="27" t="inlineStr">
         <is>
           <t>v3.39.5</t>
         </is>
       </c>
-      <c r="G63" s="24" t="inlineStr">
+      <c r="G63" s="27" t="inlineStr">
         <is>
           <t>Tokens --rhythm-sm/md/lg aplicados em main.css</t>
         </is>
       </c>
-      <c r="H63" s="24" t="inlineStr">
+      <c r="H63" s="27" t="inlineStr">
         <is>
           <t>1. Abrir src/css/main.css
 2. Grep 'var(--rhythm-' — contar
 3. Inspecionar card gaps/paddings em runtime</t>
         </is>
       </c>
-      <c r="I63" s="24" t="inlineStr">
+      <c r="I63" s="27" t="inlineStr">
         <is>
           <t>Ritmo vertical usa --rhythm-sm/md/lg consistentemente; espacamentos visualmente escalonados</t>
         </is>
       </c>
-      <c r="J63" s="24" t="inlineStr">
+      <c r="J63" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F6 + main.css</t>
         </is>
       </c>
-      <c r="K63" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L63" s="24" t="n"/>
-      <c r="M63" s="24" t="n"/>
+      <c r="K63" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L63" s="27" t="n"/>
+      <c r="M63" s="27" t="n"/>
     </row>
     <row r="64" ht="45.75" customHeight="1" s="18">
       <c r="A64" s="26" t="n">
@@ -4650,62 +4700,62 @@
       <c r="M64" s="26" t="n"/>
     </row>
     <row r="65" ht="45" customHeight="1" s="18">
-      <c r="A65" s="24" t="n">
+      <c r="A65" s="27" t="n">
         <v>63</v>
       </c>
-      <c r="B65" s="24" t="inlineStr">
+      <c r="B65" s="27" t="inlineStr">
         <is>
           <t>TC-SPC-04</t>
         </is>
       </c>
-      <c r="C65" s="24" t="inlineStr">
+      <c r="C65" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D65" s="24" t="inlineStr">
+      <c r="D65" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E65" s="24" t="inlineStr">
+      <c r="E65" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F65" s="24" t="inlineStr">
+      <c r="F65" s="27" t="inlineStr">
         <is>
           <t>v3.39.5</t>
         </is>
       </c>
-      <c r="G65" s="24" t="inlineStr">
+      <c r="G65" s="27" t="inlineStr">
         <is>
           <t>Mobile &lt;414px — spacing sobrescrito para tokens menores</t>
         </is>
       </c>
-      <c r="H65" s="24" t="inlineStr">
+      <c r="H65" s="27" t="inlineStr">
         <is>
           <t>1. DevTools responsive mode 414px ou menos
 2. Observar gaps e paddings</t>
         </is>
       </c>
-      <c r="I65" s="24" t="inlineStr">
+      <c r="I65" s="27" t="inlineStr">
         <is>
           <t>Tokens se ajustam para valores menores (media query mobile); touch targets &gt;= 44px mantidos</t>
         </is>
       </c>
-      <c r="J65" s="24" t="inlineStr">
+      <c r="J65" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F6 + mobile overrides</t>
         </is>
       </c>
-      <c r="K65" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L65" s="24" t="n"/>
-      <c r="M65" s="24" t="n"/>
+      <c r="K65" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L65" s="27" t="n"/>
+      <c r="M65" s="27" t="n"/>
     </row>
     <row r="66" ht="45.75" customHeight="1" s="18">
       <c r="A66" s="26" t="n">
@@ -4767,63 +4817,63 @@
       <c r="M66" s="26" t="n"/>
     </row>
     <row r="67" ht="45.75" customHeight="1" s="18">
-      <c r="A67" s="24" t="n">
+      <c r="A67" s="27" t="n">
         <v>65</v>
       </c>
-      <c r="B67" s="24" t="inlineStr">
+      <c r="B67" s="27" t="inlineStr">
         <is>
           <t>TC-CHART-01</t>
         </is>
       </c>
-      <c r="C67" s="24" t="inlineStr">
+      <c r="C67" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D67" s="24" t="inlineStr">
+      <c r="D67" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E67" s="24" t="inlineStr">
+      <c r="E67" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F67" s="24" t="inlineStr">
+      <c r="F67" s="27" t="inlineStr">
         <is>
           <t>v3.39.6</t>
         </is>
       </c>
-      <c r="G67" s="24" t="inlineStr">
+      <c r="G67" s="27" t="inlineStr">
         <is>
           <t>chartDefaults.js le tokens --font-size-chart-*</t>
         </is>
       </c>
-      <c r="H67" s="24" t="inlineStr">
+      <c r="H67" s="27" t="inlineStr">
         <is>
           <t>1. Abrir src/js/utils/chartDefaults.js
 2. Verificar que le CSS vars via getComputedStyle
 3. Abrir dashboard, inspecionar chart labels</t>
         </is>
       </c>
-      <c r="I67" s="24" t="inlineStr">
+      <c r="I67" s="27" t="inlineStr">
         <is>
           <t>Tipografia dos graficos respeita tokens --font-size-chart-tick/legend e --fw-chart</t>
         </is>
       </c>
-      <c r="J67" s="24" t="inlineStr">
+      <c r="J67" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F7 PR #199</t>
         </is>
       </c>
-      <c r="K67" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L67" s="24" t="n"/>
-      <c r="M67" s="24" t="n"/>
+      <c r="K67" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L67" s="27" t="n"/>
+      <c r="M67" s="27" t="n"/>
     </row>
     <row r="68" ht="45" customHeight="1" s="18">
       <c r="A68" s="26" t="n">
@@ -4884,62 +4934,62 @@
       <c r="M68" s="26" t="n"/>
     </row>
     <row r="69" ht="45" customHeight="1" s="18">
-      <c r="A69" s="24" t="n">
+      <c r="A69" s="27" t="n">
         <v>67</v>
       </c>
-      <c r="B69" s="24" t="inlineStr">
+      <c r="B69" s="27" t="inlineStr">
         <is>
           <t>TC-CHART-03</t>
         </is>
       </c>
-      <c r="C69" s="24" t="inlineStr">
+      <c r="C69" s="27" t="inlineStr">
         <is>
           <t>Design System</t>
         </is>
       </c>
-      <c r="D69" s="24" t="inlineStr">
+      <c r="D69" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E69" s="24" t="inlineStr">
+      <c r="E69" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F69" s="24" t="inlineStr">
+      <c r="F69" s="27" t="inlineStr">
         <is>
           <t>v3.39.6</t>
         </is>
       </c>
-      <c r="G69" s="24" t="inlineStr">
+      <c r="G69" s="27" t="inlineStr">
         <is>
           <t>Node.js compat — getComputedStyle fallback</t>
         </is>
       </c>
-      <c r="H69" s="24" t="inlineStr">
+      <c r="H69" s="27" t="inlineStr">
         <is>
           <t>1. Rodar npm test -- chartDefaults
 2. Verificar testes de fallback passam</t>
         </is>
       </c>
-      <c r="I69" s="24" t="inlineStr">
+      <c r="I69" s="27" t="inlineStr">
         <is>
           <t>Testes unitarios cobrem caso de SSR/Node sem window; fallback retorna valores default</t>
         </is>
       </c>
-      <c r="J69" s="24" t="inlineStr">
+      <c r="J69" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F7 + testes chartDefaults</t>
         </is>
       </c>
-      <c r="K69" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L69" s="24" t="n"/>
-      <c r="M69" s="24" t="n"/>
+      <c r="K69" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L69" s="27" t="n"/>
+      <c r="M69" s="27" t="n"/>
     </row>
     <row r="70" ht="45.75" customHeight="1" s="18">
       <c r="A70" s="26" t="n">
@@ -5001,62 +5051,62 @@
       <c r="M70" s="26" t="n"/>
     </row>
     <row r="71" ht="45" customHeight="1" s="18">
-      <c r="A71" s="24" t="n">
+      <c r="A71" s="27" t="n">
         <v>69</v>
       </c>
-      <c r="B71" s="24" t="inlineStr">
+      <c r="B71" s="27" t="inlineStr">
         <is>
           <t>TC-UX-01</t>
         </is>
       </c>
-      <c r="C71" s="24" t="inlineStr">
+      <c r="C71" s="27" t="inlineStr">
         <is>
           <t>Seguranca/UX</t>
         </is>
       </c>
-      <c r="D71" s="25" t="inlineStr">
+      <c r="D71" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E71" s="24" t="inlineStr">
+      <c r="E71" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F71" s="24" t="inlineStr">
+      <c r="F71" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G71" s="24" t="inlineStr">
+      <c r="G71" s="27" t="inlineStr">
         <is>
           <t>Zero alert() em src/</t>
         </is>
       </c>
-      <c r="H71" s="24" t="inlineStr">
+      <c r="H71" s="27" t="inlineStr">
         <is>
           <t>1. Rodar grep -rn 'alert(' src/
 2. Verificar contagem</t>
         </is>
       </c>
-      <c r="I71" s="24" t="inlineStr">
+      <c r="I71" s="27" t="inlineStr">
         <is>
           <t>Zero ocorrencias de alert() em src/js/ ou src/*.html</t>
         </is>
       </c>
-      <c r="J71" s="24" t="inlineStr">
+      <c r="J71" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 PR #200</t>
         </is>
       </c>
-      <c r="K71" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L71" s="24" t="n"/>
-      <c r="M71" s="24" t="n"/>
+      <c r="K71" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L71" s="27" t="n"/>
+      <c r="M71" s="27" t="n"/>
     </row>
     <row r="72" ht="60" customHeight="1" s="18">
       <c r="A72" s="26" t="n">
@@ -5072,7 +5122,7 @@
           <t>Transacoes/Receitas</t>
         </is>
       </c>
-      <c r="D72" s="25" t="inlineStr">
+      <c r="D72" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -5119,40 +5169,40 @@
       <c r="M72" s="26" t="n"/>
     </row>
     <row r="73" ht="60" customHeight="1" s="18">
-      <c r="A73" s="24" t="n">
+      <c r="A73" s="27" t="n">
         <v>71</v>
       </c>
-      <c r="B73" s="24" t="inlineStr">
+      <c r="B73" s="27" t="inlineStr">
         <is>
           <t>TC-UX-03</t>
         </is>
       </c>
-      <c r="C73" s="24" t="inlineStr">
+      <c r="C73" s="27" t="inlineStr">
         <is>
           <t>Config/Contas</t>
         </is>
       </c>
-      <c r="D73" s="25" t="inlineStr">
+      <c r="D73" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E73" s="24" t="inlineStr">
+      <c r="E73" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F73" s="24" t="inlineStr">
+      <c r="F73" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G73" s="24" t="inlineStr">
+      <c r="G73" s="27" t="inlineStr">
         <is>
           <t>Modal #saldo-modal-erro e #cartao-modal-erro</t>
         </is>
       </c>
-      <c r="H73" s="24" t="inlineStr">
+      <c r="H73" s="27" t="inlineStr">
         <is>
           <t>1. Config &gt; Contas
 2. Submeter alteracao de saldo invalida
@@ -5160,23 +5210,23 @@
 4. Repetir com cartao invalido</t>
         </is>
       </c>
-      <c r="I73" s="24" t="inlineStr">
+      <c r="I73" s="27" t="inlineStr">
         <is>
           <t>Ambos modais exibem erro especifico; fecham corretamente</t>
         </is>
       </c>
-      <c r="J73" s="24" t="inlineStr">
+      <c r="J73" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 + contas.html/js</t>
         </is>
       </c>
-      <c r="K73" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L73" s="24" t="n"/>
-      <c r="M73" s="24" t="n"/>
+      <c r="K73" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L73" s="27" t="n"/>
+      <c r="M73" s="27" t="n"/>
     </row>
     <row r="74" ht="45.75" customHeight="1" s="18">
       <c r="A74" s="26" t="n">
@@ -5192,7 +5242,7 @@
           <t>Historico/Patrimonio</t>
         </is>
       </c>
-      <c r="D74" s="25" t="inlineStr">
+      <c r="D74" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
@@ -5238,62 +5288,62 @@
       <c r="M74" s="26" t="n"/>
     </row>
     <row r="75" ht="45" customHeight="1" s="18">
-      <c r="A75" s="24" t="n">
+      <c r="A75" s="27" t="n">
         <v>73</v>
       </c>
-      <c r="B75" s="24" t="inlineStr">
+      <c r="B75" s="27" t="inlineStr">
         <is>
           <t>TC-UX-05</t>
         </is>
       </c>
-      <c r="C75" s="24" t="inlineStr">
+      <c r="C75" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Despesas</t>
         </is>
       </c>
-      <c r="D75" s="25" t="inlineStr">
+      <c r="D75" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E75" s="24" t="inlineStr">
+      <c r="E75" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F75" s="24" t="inlineStr">
+      <c r="F75" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G75" s="24" t="inlineStr">
+      <c r="G75" s="27" t="inlineStr">
         <is>
           <t>Empty state de Despesas com mes dinamico</t>
         </is>
       </c>
-      <c r="H75" s="24" t="inlineStr">
+      <c r="H75" s="27" t="inlineStr">
         <is>
           <t>1. Despesas em um mes vazio (sem registros)
 2. Observar empty state</t>
         </is>
       </c>
-      <c r="I75" s="24" t="inlineStr">
+      <c r="I75" s="27" t="inlineStr">
         <is>
           <t>Texto 'Sem despesas em {Mes/Ano}' substitui mensagem generica; CTA para adicionar despesa</t>
         </is>
       </c>
-      <c r="J75" s="24" t="inlineStr">
+      <c r="J75" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 + despesas.js + MF_Microcopy.md</t>
         </is>
       </c>
-      <c r="K75" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L75" s="24" t="n"/>
-      <c r="M75" s="24" t="n"/>
+      <c r="K75" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L75" s="27" t="n"/>
+      <c r="M75" s="27" t="n"/>
     </row>
     <row r="76" ht="45" customHeight="1" s="18">
       <c r="A76" s="26" t="n">
@@ -5354,62 +5404,62 @@
       <c r="M76" s="26" t="n"/>
     </row>
     <row r="77" ht="45" customHeight="1" s="18">
-      <c r="A77" s="24" t="n">
+      <c r="A77" s="27" t="n">
         <v>75</v>
       </c>
-      <c r="B77" s="24" t="inlineStr">
+      <c r="B77" s="27" t="inlineStr">
         <is>
           <t>TC-UX-07</t>
         </is>
       </c>
-      <c r="C77" s="24" t="inlineStr">
+      <c r="C77" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Fatura</t>
         </is>
       </c>
-      <c r="D77" s="24" t="inlineStr">
+      <c r="D77" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E77" s="24" t="inlineStr">
+      <c r="E77" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F77" s="24" t="inlineStr">
+      <c r="F77" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G77" s="24" t="inlineStr">
+      <c r="G77" s="27" t="inlineStr">
         <is>
           <t>Empty state de Fatura</t>
         </is>
       </c>
-      <c r="H77" s="24" t="inlineStr">
+      <c r="H77" s="27" t="inlineStr">
         <is>
           <t>1. Selecionar cartao sem fatura no mes
 2. Observar empty state</t>
         </is>
       </c>
-      <c r="I77" s="24" t="inlineStr">
+      <c r="I77" s="27" t="inlineStr">
         <is>
           <t>Mensagem contextual (cartao + mes); sem jargao tecnico</t>
         </is>
       </c>
-      <c r="J77" s="24" t="inlineStr">
+      <c r="J77" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 + fatura.js</t>
         </is>
       </c>
-      <c r="K77" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L77" s="24" t="n"/>
-      <c r="M77" s="24" t="n"/>
+      <c r="K77" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L77" s="27" t="n"/>
+      <c r="M77" s="27" t="n"/>
     </row>
     <row r="78" ht="45" customHeight="1" s="18">
       <c r="A78" s="26" t="n">
@@ -5470,62 +5520,62 @@
       <c r="M78" s="26" t="n"/>
     </row>
     <row r="79" ht="45" customHeight="1" s="18">
-      <c r="A79" s="24" t="n">
+      <c r="A79" s="27" t="n">
         <v>77</v>
       </c>
-      <c r="B79" s="24" t="inlineStr">
+      <c r="B79" s="27" t="inlineStr">
         <is>
           <t>TC-UX-09</t>
         </is>
       </c>
-      <c r="C79" s="24" t="inlineStr">
+      <c r="C79" s="27" t="inlineStr">
         <is>
           <t>Transacoes/Importar</t>
         </is>
       </c>
-      <c r="D79" s="24" t="inlineStr">
+      <c r="D79" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E79" s="24" t="inlineStr">
+      <c r="E79" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F79" s="24" t="inlineStr">
+      <c r="F79" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G79" s="24" t="inlineStr">
+      <c r="G79" s="27" t="inlineStr">
         <is>
           <t>mostrarErroUI substitui alert em falhas de import</t>
         </is>
       </c>
-      <c r="H79" s="24" t="inlineStr">
+      <c r="H79" s="27" t="inlineStr">
         <is>
           <t>1. Importar arquivo corrompido/vazio
 2. Observar feedback de erro</t>
         </is>
       </c>
-      <c r="I79" s="24" t="inlineStr">
+      <c r="I79" s="27" t="inlineStr">
         <is>
           <t>Erro via toast/modal nao-bloqueante; mensagem clara; sem alert() nativo</t>
         </is>
       </c>
-      <c r="J79" s="24" t="inlineStr">
+      <c r="J79" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 + importar.js + mostrarErroUI</t>
         </is>
       </c>
-      <c r="K79" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L79" s="24" t="n"/>
-      <c r="M79" s="24" t="n"/>
+      <c r="K79" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L79" s="27" t="n"/>
+      <c r="M79" s="27" t="n"/>
     </row>
     <row r="80" ht="45" customHeight="1" s="18">
       <c r="A80" s="26" t="n">
@@ -5586,62 +5636,62 @@
       <c r="M80" s="26" t="n"/>
     </row>
     <row r="81" ht="45" customHeight="1" s="18">
-      <c r="A81" s="24" t="n">
+      <c r="A81" s="27" t="n">
         <v>79</v>
       </c>
-      <c r="B81" s="24" t="inlineStr">
+      <c r="B81" s="27" t="inlineStr">
         <is>
           <t>TC-UX-11</t>
         </is>
       </c>
-      <c r="C81" s="24" t="inlineStr">
+      <c r="C81" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Planejamento</t>
         </is>
       </c>
-      <c r="D81" s="24" t="inlineStr">
+      <c r="D81" s="27" t="inlineStr">
         <is>
           <t>P1</t>
         </is>
       </c>
-      <c r="E81" s="24" t="inlineStr">
+      <c r="E81" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F81" s="24" t="inlineStr">
+      <c r="F81" s="27" t="inlineStr">
         <is>
           <t>v3.39.7</t>
         </is>
       </c>
-      <c r="G81" s="24" t="inlineStr">
+      <c r="G81" s="27" t="inlineStr">
         <is>
           <t>mostrarFeedback em planejamento — geracao e exclusao</t>
         </is>
       </c>
-      <c r="H81" s="24" t="inlineStr">
+      <c r="H81" s="27" t="inlineStr">
         <is>
           <t>1. Planejamento &gt; tentar gerar plano com erro
 2. Tentar excluir item com erro</t>
         </is>
       </c>
-      <c r="I81" s="24" t="inlineStr">
+      <c r="I81" s="27" t="inlineStr">
         <is>
           <t>Toast de erro em ambos casos; fluxo preservado</t>
         </is>
       </c>
-      <c r="J81" s="24" t="inlineStr">
+      <c r="J81" s="27" t="inlineStr">
         <is>
           <t>NRF-UX F8 + planejamento.js</t>
         </is>
       </c>
-      <c r="K81" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L81" s="24" t="n"/>
-      <c r="M81" s="24" t="n"/>
+      <c r="K81" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L81" s="27" t="n"/>
+      <c r="M81" s="27" t="n"/>
     </row>
     <row r="82" ht="45.75" customHeight="1" s="18">
       <c r="A82" s="26" t="n">
@@ -5703,40 +5753,40 @@
       <c r="M82" s="26" t="n"/>
     </row>
     <row r="83" ht="60" customHeight="1" s="18">
-      <c r="A83" s="24" t="n">
+      <c r="A83" s="27" t="n">
         <v>81</v>
       </c>
-      <c r="B83" s="24" t="inlineStr">
+      <c r="B83" s="27" t="inlineStr">
         <is>
           <t>TC-CTRL-01</t>
         </is>
       </c>
-      <c r="C83" s="24" t="inlineStr">
+      <c r="C83" s="27" t="inlineStr">
         <is>
           <t>Config/Categorias</t>
         </is>
       </c>
-      <c r="D83" s="24" t="inlineStr">
+      <c r="D83" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E83" s="24" t="inlineStr">
+      <c r="E83" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F83" s="24" t="inlineStr">
+      <c r="F83" s="27" t="inlineStr">
         <is>
           <t>v3.39.8</t>
         </is>
       </c>
-      <c r="G83" s="24" t="inlineStr">
+      <c r="G83" s="27" t="inlineStr">
         <is>
           <t>Criar categoria com emoji (smoke pos-refactor controller)</t>
         </is>
       </c>
-      <c r="H83" s="24" t="inlineStr">
+      <c r="H83" s="27" t="inlineStr">
         <is>
           <t>1. Config &gt; Categorias
 2. Criar nova com emoji
@@ -5744,23 +5794,23 @@
 4. Rodar npm test -- categorias.test</t>
         </is>
       </c>
-      <c r="I83" s="24" t="inlineStr">
+      <c r="I83" s="27" t="inlineStr">
         <is>
           <t>CRUD funcional; 16 testes unitarios passam</t>
         </is>
       </c>
-      <c r="J83" s="24" t="inlineStr">
+      <c r="J83" s="27" t="inlineStr">
         <is>
           <t>v3.39.8 PR #209 + tests/controllers/categorias.test.js</t>
         </is>
       </c>
-      <c r="K83" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L83" s="24" t="n"/>
-      <c r="M83" s="24" t="n"/>
+      <c r="K83" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L83" s="27" t="n"/>
+      <c r="M83" s="27" t="n"/>
     </row>
     <row r="84" ht="45.75" customHeight="1" s="18">
       <c r="A84" s="26" t="n">
@@ -5822,62 +5872,62 @@
       <c r="M84" s="26" t="n"/>
     </row>
     <row r="85" ht="45" customHeight="1" s="18">
-      <c r="A85" s="24" t="n">
+      <c r="A85" s="27" t="n">
         <v>83</v>
       </c>
-      <c r="B85" s="24" t="inlineStr">
+      <c r="B85" s="27" t="inlineStr">
         <is>
           <t>TC-CTRL-03</t>
         </is>
       </c>
-      <c r="C85" s="24" t="inlineStr">
+      <c r="C85" s="27" t="inlineStr">
         <is>
           <t>Cockpit/Planejamento</t>
         </is>
       </c>
-      <c r="D85" s="24" t="inlineStr">
+      <c r="D85" s="27" t="inlineStr">
         <is>
           <t>P2</t>
         </is>
       </c>
-      <c r="E85" s="24" t="inlineStr">
+      <c r="E85" s="27" t="inlineStr">
         <is>
           <t>Smoke</t>
         </is>
       </c>
-      <c r="F85" s="24" t="inlineStr">
+      <c r="F85" s="27" t="inlineStr">
         <is>
           <t>v3.39.8</t>
         </is>
       </c>
-      <c r="G85" s="24" t="inlineStr">
+      <c r="G85" s="27" t="inlineStr">
         <is>
           <t>autoMatch planejamento case-insensitive (pos-refactor)</t>
         </is>
       </c>
-      <c r="H85" s="24" t="inlineStr">
+      <c r="H85" s="27" t="inlineStr">
         <is>
           <t>1. Planejamento &gt; usar recurso de matching com nomes em caixas diferentes
 2. Rodar npm test -- planejamento.test</t>
         </is>
       </c>
-      <c r="I85" s="24" t="inlineStr">
+      <c r="I85" s="27" t="inlineStr">
         <is>
           <t>Match ignora maiusculas/minusculas; 32 testes unitarios passam</t>
         </is>
       </c>
-      <c r="J85" s="24" t="inlineStr">
+      <c r="J85" s="27" t="inlineStr">
         <is>
           <t>v3.39.8 + tests/controllers/planejamento.test.js</t>
         </is>
       </c>
-      <c r="K85" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L85" s="24" t="n"/>
-      <c r="M85" s="24" t="n"/>
+      <c r="K85" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L85" s="27" t="n"/>
+      <c r="M85" s="27" t="n"/>
     </row>
     <row r="86" ht="45" customHeight="1" s="18">
       <c r="A86" s="26" t="n">
@@ -5938,63 +5988,63 @@
       <c r="M86" s="26" t="n"/>
     </row>
     <row r="87" ht="45.75" customHeight="1" s="18">
-      <c r="A87" s="24" t="n">
+      <c r="A87" s="27" t="n">
         <v>85</v>
       </c>
-      <c r="B87" s="24" t="inlineStr">
+      <c r="B87" s="27" t="inlineStr">
         <is>
           <t>TC-REG-04</t>
         </is>
       </c>
-      <c r="C87" s="24" t="inlineStr">
+      <c r="C87" s="27" t="inlineStr">
         <is>
           <t>Regressao/Inviolaveis</t>
         </is>
       </c>
-      <c r="D87" s="25" t="inlineStr">
+      <c r="D87" s="28" t="inlineStr">
         <is>
           <t>P0</t>
         </is>
       </c>
-      <c r="E87" s="24" t="inlineStr">
+      <c r="E87" s="27" t="inlineStr">
         <is>
           <t>Critico</t>
         </is>
       </c>
-      <c r="F87" s="24" t="inlineStr">
+      <c r="F87" s="27" t="inlineStr">
         <is>
           <t>v3.39.1</t>
         </is>
       </c>
-      <c r="G87" s="24" t="inlineStr">
+      <c r="G87" s="27" t="inlineStr">
         <is>
           <t>Regra #14 — PR em src/**/*.html ou css/**/*.css exige ux-reviewer</t>
         </is>
       </c>
-      <c r="H87" s="24" t="inlineStr">
+      <c r="H87" s="27" t="inlineStr">
         <is>
           <t>1. Consultar ultimos PRs em main que tocaram src/
 2. Verificar se relatorio ux-reviewer foi anexado
 3. Se nao, ligar alerta</t>
         </is>
       </c>
-      <c r="I87" s="24" t="inlineStr">
+      <c r="I87" s="27" t="inlineStr">
         <is>
           <t>Todo PR que toca HTML/CSS ou templates innerHTML tem relatorio ux-reviewer em comentario/descricao</t>
         </is>
       </c>
-      <c r="J87" s="24" t="inlineStr">
+      <c r="J87" s="27" t="inlineStr">
         <is>
           <t>REGRA INVIOLAVEL 14 (CLAUDE.md + AGENTS.md + BUSSOLA §12.5)</t>
         </is>
       </c>
-      <c r="K87" s="24" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L87" s="24" t="n"/>
-      <c r="M87" s="24" t="n"/>
+      <c r="K87" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L87" s="27" t="n"/>
+      <c r="M87" s="27" t="n"/>
     </row>
     <row r="88" ht="110" customHeight="1" s="18">
       <c r="A88" s="27" t="n">
@@ -6117,60 +6167,18 @@
       <c r="A90" s="27" t="n">
         <v>88</v>
       </c>
-      <c r="B90" s="27" t="inlineStr">
-        <is>
-          <t>TC-EMPTY-03</t>
-        </is>
-      </c>
-      <c r="C90" s="27" t="inlineStr">
-        <is>
-          <t>Fluxo de Caixa</t>
-        </is>
-      </c>
-      <c r="D90" s="28" t="inlineStr">
-        <is>
-          <t>P1</t>
-        </is>
-      </c>
-      <c r="E90" s="27" t="inlineStr">
-        <is>
-          <t>Novo</t>
-        </is>
-      </c>
-      <c r="F90" s="27" t="inlineStr">
-        <is>
-          <t>v3.40.0</t>
-        </is>
-      </c>
-      <c r="G90" s="27" t="inlineStr">
-        <is>
-          <t>Empty state Cenario A — fluxo-caixa sem dados no ano</t>
-        </is>
-      </c>
-      <c r="H90" s="27" t="inlineStr">
-        <is>
-          <t>1. Acessar /fluxo-caixa.html
-2. Selecionar ano SEM despesas/receitas registradas
-3. Observar area principal</t>
-        </is>
-      </c>
-      <c r="I90" s="27" t="inlineStr">
-        <is>
-          <t>Empty state exibe SVG bar-chart, titulo com interpolacao do ano (ex: 'Sem movimentos em 2020'), CTA primario adaptado para 'adicionar despesa'; usa helper emptyStateHTML do skeletons.js</t>
-        </is>
-      </c>
-      <c r="J90" s="27" t="inlineStr">
-        <is>
-          <t>ENH-007</t>
-        </is>
-      </c>
-      <c r="K90" s="27" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="L90" s="27" t="n"/>
-      <c r="M90" s="27" t="n"/>
+      <c r="B90" s="37" t="n"/>
+      <c r="C90" s="37" t="n"/>
+      <c r="D90" s="37" t="n"/>
+      <c r="E90" s="37" t="n"/>
+      <c r="F90" s="37" t="n"/>
+      <c r="G90" s="37" t="n"/>
+      <c r="H90" s="37" t="n"/>
+      <c r="I90" s="37" t="n"/>
+      <c r="J90" s="37" t="n"/>
+      <c r="K90" s="37" t="n"/>
+      <c r="L90" s="37" t="n"/>
+      <c r="M90" s="38" t="n"/>
     </row>
     <row r="91" ht="110" customHeight="1" s="18">
       <c r="A91" s="27" t="n">
@@ -6765,364 +6773,524 @@
       <c r="L100" s="27" t="n"/>
       <c r="M100" s="27" t="n"/>
     </row>
-    <row r="101" ht="15" customHeight="1" s="18"/>
-    <row r="102" ht="15" customHeight="1" s="18"/>
-    <row r="103">
-      <c r="A103" s="29" t="inlineStr">
+    <row r="101" ht="130" customHeight="1" s="18">
+      <c r="A101" s="27" t="n">
+        <v>99</v>
+      </c>
+      <c r="B101" s="27" t="inlineStr">
+        <is>
+          <t>TC-FLUXO-03</t>
+        </is>
+      </c>
+      <c r="C101" s="27" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa (meses historicos)</t>
+        </is>
+      </c>
+      <c r="D101" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E101" s="27" t="inlineStr">
+        <is>
+          <t>Regressao pos-UAT</t>
+        </is>
+      </c>
+      <c r="F101" s="27" t="inlineStr">
+        <is>
+          <t>v3.40.0 (BUG-033 #216)</t>
+        </is>
+      </c>
+      <c r="G101" s="27" t="inlineStr">
+        <is>
+          <t>Navegacao entre meses historicos exibe dados e projecoes</t>
+        </is>
+      </c>
+      <c r="H101" s="27" t="inlineStr">
+        <is>
+          <t>1. Acessar /fluxo-caixa.html no mes atual
+2. Navegar para mes historico com dados conhecidos (ex: marco/2026)
+3. Validar que relatorios do periodo aparecem (saldos, entradas, saidas)
+4. Validar que projecoes mes a mes sao exibidas
+5. Navegar para outro mes historico (ex: fevereiro) e repetir validacao
+6. Retornar ao mes atual e validar que dados voltam corretamente</t>
+        </is>
+      </c>
+      <c r="I101" s="27" t="inlineStr">
+        <is>
+          <t>Em todos os meses historicos com registros: relatorios completos exibidos; projecoes mes a mes renderizadas; sem telas em branco; contexto de dados preservado ao mudar mes</t>
+        </is>
+      </c>
+      <c r="J101" s="27" t="inlineStr">
+        <is>
+          <t>BUG-033 / CLAUDE.md #3 isMovimentacaoReal / #6 grupoId</t>
+        </is>
+      </c>
+      <c r="K101" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L101" s="27" t="n"/>
+      <c r="M101" s="27" t="n"/>
+    </row>
+    <row r="102" ht="130" customHeight="1" s="18">
+      <c r="A102" s="27" t="n">
+        <v>100</v>
+      </c>
+      <c r="B102" s="27" t="inlineStr">
+        <is>
+          <t>TC-FLUXO-04</t>
+        </is>
+      </c>
+      <c r="C102" s="27" t="inlineStr">
+        <is>
+          <t>Fluxo de Caixa (UX abas)</t>
+        </is>
+      </c>
+      <c r="D102" s="28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="E102" s="27" t="inlineStr">
+        <is>
+          <t>Regressao pos-UAT</t>
+        </is>
+      </c>
+      <c r="F102" s="27" t="inlineStr">
+        <is>
+          <t>v3.40.0 (BUG-034 #217)</t>
+        </is>
+      </c>
+      <c r="G102" s="27" t="inlineStr">
+        <is>
+          <t>Click-outside fecha grupo de abas e libera navegacao</t>
+        </is>
+      </c>
+      <c r="H102" s="27" t="inlineStr">
+        <is>
+          <t>1. Acessar /fluxo-caixa.html
+2. Clicar em uma aba do grupo (ex: Compromissos ou Projecoes)
+3. Clicar em area externa ao grupo de abas (hero, corpo, outra secao)
+4. Confirmar que aba fechou
+5. Clicar em outra aba — confirmar que abre normalmente
+6. Repetir em viewport 375x812 (mobile) e 413x896 (limite ENH-006)</t>
+        </is>
+      </c>
+      <c r="I102" s="27" t="inlineStr">
+        <is>
+          <t>Aba fecha ao clicar fora em todos os viewports; navegacao entre abas livre; sem leak de listener apos navegar para outra pagina; comportamento consistente mobile + desktop</t>
+        </is>
+      </c>
+      <c r="J102" s="27" t="inlineStr">
+        <is>
+          <t>BUG-034 / CLAUDE.md #14 ux-reviewer</t>
+        </is>
+      </c>
+      <c r="K102" s="27" t="inlineStr">
+        <is>
+          <t>Nao iniciado</t>
+        </is>
+      </c>
+      <c r="L102" s="27" t="n"/>
+      <c r="M102" s="27" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="29" t="inlineStr">
         <is>
           <t>DASHBOARD DE PROGRESSO</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="30" t="inlineStr">
-        <is>
-          <t>Por Status</t>
         </is>
       </c>
     </row>
     <row r="105">
       <c r="A105" s="30" t="inlineStr">
         <is>
+          <t>Por Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" s="30" t="inlineStr">
+        <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="B105" s="30" t="inlineStr">
+      <c r="B106" s="30" t="inlineStr">
         <is>
           <t>Contagem</t>
         </is>
       </c>
-      <c r="C105" s="30" t="inlineStr">
+      <c r="C106" s="30" t="inlineStr">
         <is>
           <t>% do total</t>
         </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
-        <is>
-          <t>Nao iniciado</t>
-        </is>
-      </c>
-      <c r="B106">
-        <f>COUNTIF(K3:K100,"Nao iniciado")</f>
-        <v/>
-      </c>
-      <c r="C106" s="31">
-        <f>IFERROR(B106/98,0)</f>
-        <v/>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Em execucao</t>
+          <t>Nao iniciado</t>
         </is>
       </c>
       <c r="B107">
-        <f>COUNTIF(K3:K100,"Em execucao")</f>
+        <f>COUNTIF(K3:K102,"Nao iniciado")</f>
         <v/>
       </c>
       <c r="C107" s="31">
-        <f>IFERROR(B107/98,0)</f>
+        <f>IFERROR(B107/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>PASS</t>
+          <t>Em execucao</t>
         </is>
       </c>
       <c r="B108">
-        <f>COUNTIF(K3:K100,"PASS")</f>
+        <f>COUNTIF(K3:K102,"Em execucao")</f>
         <v/>
       </c>
       <c r="C108" s="31">
-        <f>IFERROR(B108/98,0)</f>
+        <f>IFERROR(B108/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>FAIL</t>
+          <t>PASS</t>
         </is>
       </c>
       <c r="B109">
-        <f>COUNTIF(K3:K100,"FAIL")</f>
+        <f>COUNTIF(K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C109" s="31">
-        <f>IFERROR(B109/98,0)</f>
+        <f>IFERROR(B109/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>FAIL</t>
         </is>
       </c>
       <c r="B110">
-        <f>COUNTIF(K3:K100,"N/A")</f>
+        <f>COUNTIF(K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="C110" s="31">
-        <f>IFERROR(B110/98,0)</f>
+        <f>IFERROR(B110/100,0)</f>
         <v/>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="B111">
+        <f>COUNTIF(K3:K102,"N/A")</f>
+        <v/>
+      </c>
+      <c r="C111" s="31">
+        <f>IFERROR(B111/100,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
           <t>BLOCKED</t>
         </is>
       </c>
-      <c r="B111">
-        <f>COUNTIF(K3:K100,"BLOCKED")</f>
+      <c r="B112">
+        <f>COUNTIF(K3:K102,"BLOCKED")</f>
         <v/>
       </c>
-      <c r="C111" s="31">
-        <f>IFERROR(B111/98,0)</f>
+      <c r="C112" s="31">
+        <f>IFERROR(B112/100,0)</f>
         <v/>
-      </c>
-    </row>
-    <row r="113">
-      <c r="A113" s="30" t="inlineStr">
-        <is>
-          <t>Por Origem</t>
-        </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" s="30" t="inlineStr">
         <is>
+          <t>Por Origem</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" s="30" t="inlineStr">
+        <is>
           <t>Origem</t>
         </is>
       </c>
-      <c r="B114" s="30" t="inlineStr">
+      <c r="B115" s="30" t="inlineStr">
         <is>
           <t>PASS</t>
         </is>
       </c>
-      <c r="C114" s="30" t="inlineStr">
+      <c r="C115" s="30" t="inlineStr">
         <is>
           <t>FAIL</t>
         </is>
       </c>
-      <c r="D114" s="30" t="inlineStr">
+      <c r="D115" s="30" t="inlineStr">
         <is>
           <t>Pendentes</t>
         </is>
-      </c>
-    </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
-        <is>
-          <t>v3.38.0</t>
-        </is>
-      </c>
-      <c r="B115">
-        <f>COUNTIFS(F3:F100,"v3.38.0",K3:K100,"PASS")</f>
-        <v/>
-      </c>
-      <c r="C115">
-        <f>COUNTIFS(F3:F100,"v3.38.0",K3:K100,"FAIL")</f>
-        <v/>
-      </c>
-      <c r="D115">
-        <f>COUNTIFS(F3:F100,"v3.38.0",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.38.0",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.38.0",K3:K100,"BLOCKED")</f>
-        <v/>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>v3.39.0</t>
+          <t>v3.38.0</t>
         </is>
       </c>
       <c r="B116">
-        <f>COUNTIFS(F3:F100,"v3.39.0",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.38.0",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C116">
-        <f>COUNTIFS(F3:F100,"v3.39.0",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.38.0",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D116">
-        <f>COUNTIFS(F3:F100,"v3.39.0",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.0",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.0",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.38.0",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.38.0",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.38.0",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>v3.39.1</t>
+          <t>v3.39.0</t>
         </is>
       </c>
       <c r="B117">
-        <f>COUNTIFS(F3:F100,"v3.39.1",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.0",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C117">
-        <f>COUNTIFS(F3:F100,"v3.39.1",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.0",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D117">
-        <f>COUNTIFS(F3:F100,"v3.39.1",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.1",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.1",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.0",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.0",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.0",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>v3.39.2</t>
+          <t>v3.39.1</t>
         </is>
       </c>
       <c r="B118">
-        <f>COUNTIFS(F3:F100,"v3.39.2",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.1",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C118">
-        <f>COUNTIFS(F3:F100,"v3.39.2",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.1",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D118">
-        <f>COUNTIFS(F3:F100,"v3.39.2",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.2",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.2",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.1",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.1",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.1",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>v3.39.3</t>
+          <t>v3.39.2</t>
         </is>
       </c>
       <c r="B119">
-        <f>COUNTIFS(F3:F100,"v3.39.3",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.2",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C119">
-        <f>COUNTIFS(F3:F100,"v3.39.3",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.2",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D119">
-        <f>COUNTIFS(F3:F100,"v3.39.3",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.3",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.3",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.2",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.2",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.2",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>v3.39.4</t>
+          <t>v3.39.3</t>
         </is>
       </c>
       <c r="B120">
-        <f>COUNTIFS(F3:F100,"v3.39.4",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.3",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C120">
-        <f>COUNTIFS(F3:F100,"v3.39.4",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.3",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D120">
-        <f>COUNTIFS(F3:F100,"v3.39.4",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.4",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.4",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.3",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.3",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.3",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>v3.39.5</t>
+          <t>v3.39.4</t>
         </is>
       </c>
       <c r="B121">
-        <f>COUNTIFS(F3:F100,"v3.39.5",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.4",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C121">
-        <f>COUNTIFS(F3:F100,"v3.39.5",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.4",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D121">
-        <f>COUNTIFS(F3:F100,"v3.39.5",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.5",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.5",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.4",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.4",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.4",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>v3.39.6</t>
+          <t>v3.39.5</t>
         </is>
       </c>
       <c r="B122">
-        <f>COUNTIFS(F3:F100,"v3.39.6",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.5",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C122">
-        <f>COUNTIFS(F3:F100,"v3.39.6",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.5",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D122">
-        <f>COUNTIFS(F3:F100,"v3.39.6",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.6",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.6",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.5",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.5",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.5",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>v3.39.7</t>
+          <t>v3.39.6</t>
         </is>
       </c>
       <c r="B123">
-        <f>COUNTIFS(F3:F100,"v3.39.7",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.6",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C123">
-        <f>COUNTIFS(F3:F100,"v3.39.7",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.6",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D123">
-        <f>COUNTIFS(F3:F100,"v3.39.7",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.7",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.7",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.6",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.6",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.6",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>v3.39.8</t>
+          <t>v3.39.7</t>
         </is>
       </c>
       <c r="B124">
-        <f>COUNTIFS(F3:F100,"v3.39.8",K3:K100,"PASS")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.7",K3:K102,"PASS")</f>
         <v/>
       </c>
       <c r="C124">
-        <f>COUNTIFS(F3:F100,"v3.39.8",K3:K100,"FAIL")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.7",K3:K102,"FAIL")</f>
         <v/>
       </c>
       <c r="D124">
-        <f>COUNTIFS(F3:F100,"v3.39.8",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.39.8",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.39.8",K3:K100,"BLOCKED")</f>
+        <f>COUNTIFS(F3:F102,"v3.39.7",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.7",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.7",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
+          <t>v3.39.8</t>
+        </is>
+      </c>
+      <c r="B125">
+        <f>COUNTIFS(F3:F102,"v3.39.8",K3:K102,"PASS")</f>
+        <v/>
+      </c>
+      <c r="C125">
+        <f>COUNTIFS(F3:F102,"v3.39.8",K3:K102,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="D125">
+        <f>COUNTIFS(F3:F102,"v3.39.8",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.39.8",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.39.8",K3:K102,"BLOCKED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
           <t>v3.40.0</t>
         </is>
       </c>
-      <c r="B125">
-        <f>COUNTIFS(F3:F100,"v3.40.0",K3:K100,"PASS")</f>
+      <c r="B126">
+        <f>COUNTIFS(F3:F102,"v3.40.0",K3:K102,"PASS")</f>
         <v/>
       </c>
-      <c r="C125">
-        <f>COUNTIFS(F3:F100,"v3.40.0",K3:K100,"FAIL")</f>
+      <c r="C126">
+        <f>COUNTIFS(F3:F102,"v3.40.0",K3:K102,"FAIL")</f>
         <v/>
       </c>
-      <c r="D125">
-        <f>COUNTIFS(F3:F100,"v3.40.0",K3:K100,"Nao iniciado")+COUNTIFS(F3:F100,"v3.40.0",K3:K100,"Em execucao")+COUNTIFS(F3:F100,"v3.40.0",K3:K100,"BLOCKED")</f>
+      <c r="D126">
+        <f>COUNTIFS(F3:F102,"v3.40.0",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.40.0",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.40.0",K3:K102,"BLOCKED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>v3.40.0 (BUG-033 #216)</t>
+        </is>
+      </c>
+      <c r="B127">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-033 #216)",K3:K102,"PASS")</f>
+        <v/>
+      </c>
+      <c r="C127">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-033 #216)",K3:K102,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="D127">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-033 #216)",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.40.0 (BUG-033 #216)",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.40.0 (BUG-033 #216)",K3:K102,"BLOCKED")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>v3.40.0 (BUG-034 #217)</t>
+        </is>
+      </c>
+      <c r="B128">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-034 #217)",K3:K102,"PASS")</f>
+        <v/>
+      </c>
+      <c r="C128">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-034 #217)",K3:K102,"FAIL")</f>
+        <v/>
+      </c>
+      <c r="D128">
+        <f>COUNTIFS(F3:F102,"v3.40.0 (BUG-034 #217)",K3:K102,"Nao iniciado")+COUNTIFS(F3:F102,"v3.40.0 (BUG-034 #217)",K3:K102,"Em execucao")+COUNTIFS(F3:F102,"v3.40.0 (BUG-034 #217)",K3:K102,"BLOCKED")</f>
         <v/>
       </c>
     </row>
@@ -7224,10 +7392,10 @@
       </c>
     </row>
     <row r="5" ht="15" customHeight="1" s="18">
-      <c r="A5" s="24" t="n">
+      <c r="A5" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="24" t="inlineStr">
+      <c r="B5" s="27" t="inlineStr">
         <is>
           <t>chave_dedup alterada</t>
         </is>
@@ -7237,7 +7405,7 @@
           <t>BLOQUEANTE</t>
         </is>
       </c>
-      <c r="D5" s="24" t="inlineStr">
+      <c r="D5" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7264,10 +7432,10 @@
       </c>
     </row>
     <row r="7" ht="15" customHeight="1" s="18">
-      <c r="A7" s="24" t="n">
+      <c r="A7" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="B7" s="24" t="inlineStr">
+      <c r="B7" s="27" t="inlineStr">
         <is>
           <t>isMovimentacaoReal() nao usado em agregado que filtra projecoes</t>
         </is>
@@ -7277,7 +7445,7 @@
           <t>BLOQUEANTE</t>
         </is>
       </c>
-      <c r="D7" s="24" t="inlineStr">
+      <c r="D7" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7304,10 +7472,10 @@
       </c>
     </row>
     <row r="9" ht="15" customHeight="1" s="18">
-      <c r="A9" s="24" t="n">
+      <c r="A9" s="27" t="n">
         <v>5</v>
       </c>
-      <c r="B9" s="24" t="inlineStr">
+      <c r="B9" s="27" t="inlineStr">
         <is>
           <t>Firebase via CDN gstatic.com (nao npm)</t>
         </is>
@@ -7317,7 +7485,7 @@
           <t>BLOQUEANTE</t>
         </is>
       </c>
-      <c r="D9" s="24" t="inlineStr">
+      <c r="D9" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7344,10 +7512,10 @@
       </c>
     </row>
     <row r="11" ht="15" customHeight="1" s="18">
-      <c r="A11" s="24" t="n">
+      <c r="A11" s="27" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="24" t="inlineStr">
+      <c r="B11" s="27" t="inlineStr">
         <is>
           <t>innerHTML sem escHTML() em dados do usuario</t>
         </is>
@@ -7357,7 +7525,7 @@
           <t>BLOQUEANTE</t>
         </is>
       </c>
-      <c r="D11" s="24" t="inlineStr">
+      <c r="D11" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7384,10 +7552,10 @@
       </c>
     </row>
     <row r="13" ht="15" customHeight="1" s="18">
-      <c r="A13" s="24" t="n">
+      <c r="A13" s="27" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="24" t="inlineStr">
+      <c r="B13" s="27" t="inlineStr">
         <is>
           <t>deleteDoc em lote sem writeBatch</t>
         </is>
@@ -7397,7 +7565,7 @@
           <t>BLOQUEANTE</t>
         </is>
       </c>
-      <c r="D13" s="24" t="inlineStr">
+      <c r="D13" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7424,10 +7592,10 @@
       </c>
     </row>
     <row r="15" ht="15" customHeight="1" s="18">
-      <c r="A15" s="24" t="n">
+      <c r="A15" s="27" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="24" t="inlineStr">
+      <c r="B15" s="27" t="inlineStr">
         <is>
           <t>Commit sem Conventional Commits com escopo</t>
         </is>
@@ -7437,7 +7605,7 @@
           <t>ALERTA</t>
         </is>
       </c>
-      <c r="D15" s="24" t="inlineStr">
+      <c r="D15" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>
@@ -7464,10 +7632,10 @@
       </c>
     </row>
     <row r="17" ht="15" customHeight="1" s="18">
-      <c r="A17" s="24" t="n">
+      <c r="A17" s="27" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="24" t="inlineStr">
+      <c r="B17" s="27" t="inlineStr">
         <is>
           <t>Task de UI sem consultar docs/DESIGN_SYSTEM.md / tokens</t>
         </is>
@@ -7477,7 +7645,7 @@
           <t>ALERTA</t>
         </is>
       </c>
-      <c r="D17" s="24" t="inlineStr">
+      <c r="D17" s="27" t="inlineStr">
         <is>
           <t>NAO</t>
         </is>

</xml_diff>